<commit_message>
chore(consensus): 주간 컨센 스냅샷 2026-09-28
</commit_message>
<xml_diff>
--- a/telegram_research_dashboard/static/consensus_full.xlsx
+++ b/telegram_research_dashboard/static/consensus_full.xlsx
@@ -618,7 +618,7 @@
         <v>2081.7</v>
       </c>
       <c r="U3" t="n">
-        <v>15100</v>
+        <v>15110</v>
       </c>
     </row>
     <row r="4">
@@ -684,13 +684,13 @@
         <v>0</v>
       </c>
       <c r="U4" t="n">
-        <v>74800</v>
+        <v>74400</v>
       </c>
       <c r="V4" t="n">
         <v>76000</v>
       </c>
       <c r="W4" t="n">
-        <v>-1.6</v>
+        <v>-2.1</v>
       </c>
     </row>
     <row r="5">
@@ -756,13 +756,13 @@
         <v>0</v>
       </c>
       <c r="U5" t="n">
-        <v>70500</v>
+        <v>70400</v>
       </c>
       <c r="V5" t="n">
         <v>71000</v>
       </c>
       <c r="W5" t="n">
-        <v>-0.7</v>
+        <v>-0.8</v>
       </c>
     </row>
     <row r="6">
@@ -804,7 +804,7 @@
         <v>31331</v>
       </c>
       <c r="U6" t="n">
-        <v>1433000</v>
+        <v>1415000</v>
       </c>
     </row>
     <row r="7">
@@ -846,7 +846,7 @@
         <v>6170</v>
       </c>
       <c r="U7" t="n">
-        <v>52300</v>
+        <v>51900</v>
       </c>
     </row>
     <row r="8">
@@ -954,13 +954,13 @@
         <v>0</v>
       </c>
       <c r="U9" t="n">
-        <v>116300</v>
+        <v>117100</v>
       </c>
       <c r="V9" t="n">
         <v>121600</v>
       </c>
       <c r="W9" t="n">
-        <v>-4.4</v>
+        <v>-3.7</v>
       </c>
     </row>
     <row r="10">
@@ -1026,13 +1026,13 @@
         <v>0</v>
       </c>
       <c r="U10" t="n">
-        <v>92700</v>
+        <v>93700</v>
       </c>
       <c r="V10" t="n">
         <v>93600</v>
       </c>
       <c r="W10" t="n">
-        <v>-1</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="11">
@@ -1098,13 +1098,13 @@
         <v>2.4</v>
       </c>
       <c r="U11" t="n">
-        <v>1778000</v>
+        <v>1761000</v>
       </c>
       <c r="V11" t="n">
         <v>1849000</v>
       </c>
       <c r="W11" t="n">
-        <v>-3.8</v>
+        <v>-4.8</v>
       </c>
     </row>
     <row r="12">
@@ -1170,13 +1170,13 @@
         <v>0.2</v>
       </c>
       <c r="U12" t="n">
-        <v>125100</v>
+        <v>123200</v>
       </c>
       <c r="V12" t="n">
         <v>125600</v>
       </c>
       <c r="W12" t="n">
-        <v>-0.4</v>
+        <v>-1.9</v>
       </c>
     </row>
     <row r="13">
@@ -1218,7 +1218,7 @@
         <v>37044</v>
       </c>
       <c r="U13" t="n">
-        <v>650000</v>
+        <v>658000</v>
       </c>
     </row>
     <row r="14">
@@ -1260,7 +1260,7 @@
         <v>77944.8</v>
       </c>
       <c r="U14" t="n">
-        <v>132400</v>
+        <v>131500</v>
       </c>
     </row>
     <row r="15">
@@ -1302,7 +1302,7 @@
         <v>7010</v>
       </c>
       <c r="U15" t="n">
-        <v>130100</v>
+        <v>125600</v>
       </c>
     </row>
     <row r="16">
@@ -1344,7 +1344,7 @@
         <v>30875.4</v>
       </c>
       <c r="U16" t="n">
-        <v>134900</v>
+        <v>133300</v>
       </c>
     </row>
     <row r="17">
@@ -1410,13 +1410,13 @@
         <v>0</v>
       </c>
       <c r="U17" t="n">
-        <v>45850</v>
+        <v>44750</v>
       </c>
       <c r="V17" t="n">
         <v>45150</v>
       </c>
       <c r="W17" t="n">
-        <v>1.6</v>
+        <v>-0.9</v>
       </c>
     </row>
     <row r="18">
@@ -1458,7 +1458,7 @@
         <v>3257.1</v>
       </c>
       <c r="U18" t="n">
-        <v>30350</v>
+        <v>29850</v>
       </c>
     </row>
     <row r="19">
@@ -1497,7 +1497,7 @@
         <v>15992.7</v>
       </c>
       <c r="U19" t="n">
-        <v>49000</v>
+        <v>48600</v>
       </c>
     </row>
     <row r="20">
@@ -1533,7 +1533,7 @@
         <v>2028</v>
       </c>
       <c r="U20" t="n">
-        <v>18330</v>
+        <v>18290</v>
       </c>
     </row>
     <row r="21">
@@ -1575,7 +1575,7 @@
         <v>6750</v>
       </c>
       <c r="U21" t="n">
-        <v>24050</v>
+        <v>24000</v>
       </c>
     </row>
     <row r="22">
@@ -1641,13 +1641,13 @@
         <v>0</v>
       </c>
       <c r="U22" t="n">
-        <v>5690</v>
+        <v>5730</v>
       </c>
       <c r="V22" t="n">
         <v>5580</v>
       </c>
       <c r="W22" t="n">
-        <v>2</v>
+        <v>2.7</v>
       </c>
     </row>
     <row r="23">
@@ -1689,7 +1689,7 @@
         <v>5566</v>
       </c>
       <c r="U23" t="n">
-        <v>476500</v>
+        <v>477500</v>
       </c>
     </row>
     <row r="24">
@@ -1755,13 +1755,13 @@
         <v>0</v>
       </c>
       <c r="U24" t="n">
-        <v>12900</v>
+        <v>12950</v>
       </c>
       <c r="V24" t="n">
         <v>13480</v>
       </c>
       <c r="W24" t="n">
-        <v>-4.3</v>
+        <v>-3.9</v>
       </c>
     </row>
     <row r="25">
@@ -1803,7 +1803,7 @@
         <v>3620</v>
       </c>
       <c r="U25" t="n">
-        <v>106400</v>
+        <v>107800</v>
       </c>
     </row>
     <row r="26">
@@ -1869,13 +1869,13 @@
         <v>0</v>
       </c>
       <c r="U26" t="n">
-        <v>9220</v>
+        <v>9200</v>
       </c>
       <c r="V26" t="n">
         <v>9420</v>
       </c>
       <c r="W26" t="n">
-        <v>-2.1</v>
+        <v>-2.3</v>
       </c>
     </row>
     <row r="27">
@@ -2013,13 +2013,13 @@
         <v>0</v>
       </c>
       <c r="U28" t="n">
-        <v>1220000</v>
+        <v>1218000</v>
       </c>
       <c r="V28" t="n">
         <v>1296000</v>
       </c>
       <c r="W28" t="n">
-        <v>-5.9</v>
+        <v>-6</v>
       </c>
     </row>
     <row r="29">
@@ -2199,13 +2199,13 @@
         <v>-0.1</v>
       </c>
       <c r="U31" t="n">
-        <v>182000</v>
+        <v>182600</v>
       </c>
       <c r="V31" t="n">
         <v>183300</v>
       </c>
       <c r="W31" t="n">
-        <v>-0.7</v>
+        <v>-0.4</v>
       </c>
     </row>
     <row r="32">
@@ -2247,7 +2247,7 @@
         <v>1807.7</v>
       </c>
       <c r="U32" t="n">
-        <v>43700</v>
+        <v>44000</v>
       </c>
     </row>
     <row r="33">
@@ -2313,13 +2313,13 @@
         <v>-0.7</v>
       </c>
       <c r="U33" t="n">
-        <v>30800</v>
+        <v>31000</v>
       </c>
       <c r="V33" t="n">
         <v>35850</v>
       </c>
       <c r="W33" t="n">
-        <v>-14.1</v>
+        <v>-13.5</v>
       </c>
     </row>
     <row r="34">
@@ -2361,7 +2361,7 @@
         <v>9348.6</v>
       </c>
       <c r="U34" t="n">
-        <v>349000</v>
+        <v>343000</v>
       </c>
     </row>
     <row r="35">
@@ -2427,13 +2427,13 @@
         <v>0</v>
       </c>
       <c r="U35" t="n">
-        <v>394000</v>
+        <v>394500</v>
       </c>
       <c r="V35" t="n">
         <v>392500</v>
       </c>
       <c r="W35" t="n">
-        <v>0.4</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="36">
@@ -2475,7 +2475,7 @@
         <v>5355</v>
       </c>
       <c r="U36" t="n">
-        <v>24450</v>
+        <v>24650</v>
       </c>
     </row>
     <row r="37">
@@ -2541,13 +2541,13 @@
         <v>0</v>
       </c>
       <c r="U37" t="n">
-        <v>95700</v>
+        <v>96000</v>
       </c>
       <c r="V37" t="n">
         <v>94600</v>
       </c>
       <c r="W37" t="n">
-        <v>1.2</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="38">
@@ -2613,13 +2613,13 @@
         <v>0</v>
       </c>
       <c r="U38" t="n">
-        <v>354500</v>
+        <v>354000</v>
       </c>
       <c r="V38" t="n">
         <v>366500</v>
       </c>
       <c r="W38" t="n">
-        <v>-3.3</v>
+        <v>-3.4</v>
       </c>
     </row>
     <row r="39">
@@ -2685,13 +2685,13 @@
         <v>0</v>
       </c>
       <c r="U39" t="n">
-        <v>315500</v>
+        <v>313500</v>
       </c>
       <c r="V39" t="n">
         <v>325500</v>
       </c>
       <c r="W39" t="n">
-        <v>-3.1</v>
+        <v>-3.7</v>
       </c>
     </row>
     <row r="40">
@@ -2730,7 +2730,7 @@
         <v>25469.6</v>
       </c>
       <c r="U40" t="n">
-        <v>187200</v>
+        <v>190300</v>
       </c>
     </row>
     <row r="41">
@@ -2796,13 +2796,13 @@
         <v>0</v>
       </c>
       <c r="U41" t="n">
-        <v>50100</v>
+        <v>50300</v>
       </c>
       <c r="V41" t="n">
         <v>50400</v>
       </c>
       <c r="W41" t="n">
-        <v>-0.6</v>
+        <v>-0.2</v>
       </c>
     </row>
     <row r="42">
@@ -2868,13 +2868,13 @@
         <v>3.3</v>
       </c>
       <c r="U42" t="n">
-        <v>274500</v>
+        <v>270000</v>
       </c>
       <c r="V42" t="n">
         <v>260000</v>
       </c>
       <c r="W42" t="n">
-        <v>5.6</v>
+        <v>3.8</v>
       </c>
     </row>
     <row r="43">
@@ -2982,13 +2982,13 @@
         <v>0</v>
       </c>
       <c r="U44" t="n">
-        <v>8390</v>
+        <v>8440</v>
       </c>
       <c r="V44" t="n">
         <v>8670</v>
       </c>
       <c r="W44" t="n">
-        <v>-3.2</v>
+        <v>-2.7</v>
       </c>
     </row>
     <row r="45">
@@ -3054,13 +3054,13 @@
         <v>0</v>
       </c>
       <c r="U45" t="n">
-        <v>35700</v>
+        <v>36000</v>
       </c>
       <c r="V45" t="n">
         <v>35750</v>
       </c>
       <c r="W45" t="n">
-        <v>-0.1</v>
+        <v>0.7</v>
       </c>
     </row>
     <row r="46">
@@ -3102,7 +3102,7 @@
         <v>26635.8</v>
       </c>
       <c r="U46" t="n">
-        <v>314500</v>
+        <v>312000</v>
       </c>
     </row>
     <row r="47">
@@ -3168,13 +3168,13 @@
         <v>0</v>
       </c>
       <c r="U47" t="n">
-        <v>123200</v>
+        <v>122900</v>
       </c>
       <c r="V47" t="n">
         <v>122100</v>
       </c>
       <c r="W47" t="n">
-        <v>0.9</v>
+        <v>0.7</v>
       </c>
     </row>
     <row r="48">
@@ -3240,13 +3240,13 @@
         <v>0.3</v>
       </c>
       <c r="U48" t="n">
-        <v>35750</v>
+        <v>35350</v>
       </c>
       <c r="V48" t="n">
         <v>37200</v>
       </c>
       <c r="W48" t="n">
-        <v>-3.9</v>
+        <v>-5</v>
       </c>
     </row>
     <row r="49">
@@ -3312,13 +3312,13 @@
         <v>-0.9</v>
       </c>
       <c r="U49" t="n">
-        <v>531000</v>
+        <v>528000</v>
       </c>
       <c r="V49" t="n">
         <v>542000</v>
       </c>
       <c r="W49" t="n">
-        <v>-2</v>
+        <v>-2.6</v>
       </c>
     </row>
     <row r="50">
@@ -3360,7 +3360,7 @@
         <v>2380.2</v>
       </c>
       <c r="U50" t="n">
-        <v>92600</v>
+        <v>91800</v>
       </c>
     </row>
     <row r="51">
@@ -3402,7 +3402,7 @@
         <v>27610.4</v>
       </c>
       <c r="U51" t="n">
-        <v>31700</v>
+        <v>31650</v>
       </c>
     </row>
     <row r="52">
@@ -3444,7 +3444,7 @@
         <v>4117.4</v>
       </c>
       <c r="U52" t="n">
-        <v>22950</v>
+        <v>23050</v>
       </c>
     </row>
     <row r="53">
@@ -3486,7 +3486,7 @@
         <v>8137</v>
       </c>
       <c r="U53" t="n">
-        <v>48950</v>
+        <v>50400</v>
       </c>
     </row>
     <row r="54">
@@ -3552,13 +3552,13 @@
         <v>0.7</v>
       </c>
       <c r="U54" t="n">
-        <v>115300</v>
+        <v>112000</v>
       </c>
       <c r="V54" t="n">
         <v>102400</v>
       </c>
       <c r="W54" t="n">
-        <v>12.6</v>
+        <v>9.4</v>
       </c>
     </row>
     <row r="55">
@@ -3624,13 +3624,13 @@
         <v>0</v>
       </c>
       <c r="U55" t="n">
-        <v>69300</v>
+        <v>69600</v>
       </c>
       <c r="V55" t="n">
         <v>52200</v>
       </c>
       <c r="W55" t="n">
-        <v>32.8</v>
+        <v>33.3</v>
       </c>
     </row>
     <row r="56">
@@ -3672,7 +3672,7 @@
         <v>2727.2</v>
       </c>
       <c r="U56" t="n">
-        <v>40200</v>
+        <v>40300</v>
       </c>
     </row>
     <row r="57">
@@ -3738,13 +3738,13 @@
         <v>0.3</v>
       </c>
       <c r="U57" t="n">
-        <v>1503000</v>
+        <v>1491000</v>
       </c>
       <c r="V57" t="n">
         <v>1388000</v>
       </c>
       <c r="W57" t="n">
-        <v>8.300000000000001</v>
+        <v>7.4</v>
       </c>
     </row>
     <row r="58">
@@ -3786,7 +3786,7 @@
         <v>536.8</v>
       </c>
       <c r="U58" t="n">
-        <v>40650</v>
+        <v>40400</v>
       </c>
     </row>
     <row r="59">
@@ -3900,7 +3900,7 @@
         <v>14592.8</v>
       </c>
       <c r="U60" t="n">
-        <v>32500</v>
+        <v>34250</v>
       </c>
     </row>
     <row r="61">
@@ -3942,7 +3942,7 @@
         <v>6588.9</v>
       </c>
       <c r="U61" t="n">
-        <v>226500</v>
+        <v>232000</v>
       </c>
     </row>
     <row r="62">
@@ -4008,13 +4008,13 @@
         <v>0</v>
       </c>
       <c r="U62" t="n">
-        <v>204000</v>
+        <v>203000</v>
       </c>
       <c r="V62" t="n">
         <v>208500</v>
       </c>
       <c r="W62" t="n">
-        <v>-2.2</v>
+        <v>-2.6</v>
       </c>
     </row>
     <row r="63">
@@ -4080,13 +4080,13 @@
         <v>0</v>
       </c>
       <c r="U63" t="n">
-        <v>1105000</v>
+        <v>1094000</v>
       </c>
       <c r="V63" t="n">
         <v>1132000</v>
       </c>
       <c r="W63" t="n">
-        <v>-2.4</v>
+        <v>-3.4</v>
       </c>
     </row>
     <row r="64">
@@ -4191,7 +4191,7 @@
         <v>59</v>
       </c>
       <c r="U65" t="n">
-        <v>17600</v>
+        <v>17260</v>
       </c>
     </row>
     <row r="66">
@@ -4257,7 +4257,7 @@
         <v>0</v>
       </c>
       <c r="U66" t="n">
-        <v>14980</v>
+        <v>14970</v>
       </c>
       <c r="V66" t="n">
         <v>15500</v>
@@ -4305,7 +4305,7 @@
         <v>28485.6</v>
       </c>
       <c r="U67" t="n">
-        <v>163300</v>
+        <v>164000</v>
       </c>
     </row>
     <row r="68">
@@ -4371,13 +4371,13 @@
         <v>-0.8</v>
       </c>
       <c r="U68" t="n">
-        <v>579000</v>
+        <v>574000</v>
       </c>
       <c r="V68" t="n">
         <v>531000</v>
       </c>
       <c r="W68" t="n">
-        <v>9</v>
+        <v>8.1</v>
       </c>
     </row>
     <row r="69">
@@ -4419,7 +4419,7 @@
         <v>3593.9</v>
       </c>
       <c r="U69" t="n">
-        <v>61700</v>
+        <v>62400</v>
       </c>
     </row>
     <row r="70">
@@ -4485,13 +4485,13 @@
         <v>0</v>
       </c>
       <c r="U70" t="n">
-        <v>21200</v>
+        <v>21350</v>
       </c>
       <c r="V70" t="n">
         <v>20950</v>
       </c>
       <c r="W70" t="n">
-        <v>1.2</v>
+        <v>1.9</v>
       </c>
     </row>
     <row r="71">
@@ -4557,13 +4557,13 @@
         <v>0</v>
       </c>
       <c r="U71" t="n">
-        <v>54200</v>
+        <v>53500</v>
       </c>
       <c r="V71" t="n">
         <v>54700</v>
       </c>
       <c r="W71" t="n">
-        <v>-0.9</v>
+        <v>-2.2</v>
       </c>
     </row>
     <row r="72">
@@ -4605,7 +4605,7 @@
         <v>4720.3</v>
       </c>
       <c r="U72" t="n">
-        <v>118600</v>
+        <v>117500</v>
       </c>
     </row>
     <row r="73">
@@ -4647,7 +4647,7 @@
         <v>2495</v>
       </c>
       <c r="U73" t="n">
-        <v>91200</v>
+        <v>90200</v>
       </c>
     </row>
     <row r="74">
@@ -4713,13 +4713,13 @@
         <v>0</v>
       </c>
       <c r="U74" t="n">
-        <v>17660</v>
+        <v>17700</v>
       </c>
       <c r="V74" t="n">
         <v>16960</v>
       </c>
       <c r="W74" t="n">
-        <v>4.1</v>
+        <v>4.4</v>
       </c>
     </row>
     <row r="75">
@@ -4785,13 +4785,13 @@
         <v>0</v>
       </c>
       <c r="U75" t="n">
-        <v>374500</v>
+        <v>371500</v>
       </c>
       <c r="V75" t="n">
         <v>380500</v>
       </c>
       <c r="W75" t="n">
-        <v>-1.6</v>
+        <v>-2.4</v>
       </c>
     </row>
     <row r="76">
@@ -4857,13 +4857,13 @@
         <v>0</v>
       </c>
       <c r="U76" t="n">
-        <v>1043000</v>
+        <v>1034000</v>
       </c>
       <c r="V76" t="n">
         <v>1092000</v>
       </c>
       <c r="W76" t="n">
-        <v>-4.5</v>
+        <v>-5.3</v>
       </c>
     </row>
     <row r="77">
@@ -4905,7 +4905,7 @@
         <v>2558.3</v>
       </c>
       <c r="U77" t="n">
-        <v>335500</v>
+        <v>332000</v>
       </c>
     </row>
     <row r="78">
@@ -4947,7 +4947,7 @@
         <v>2694</v>
       </c>
       <c r="U78" t="n">
-        <v>82300</v>
+        <v>82900</v>
       </c>
     </row>
     <row r="79">
@@ -5013,13 +5013,13 @@
         <v>0</v>
       </c>
       <c r="U79" t="n">
-        <v>31200</v>
+        <v>31150</v>
       </c>
       <c r="V79" t="n">
         <v>32300</v>
       </c>
       <c r="W79" t="n">
-        <v>-3.4</v>
+        <v>-3.6</v>
       </c>
     </row>
     <row r="80">
@@ -5085,13 +5085,13 @@
         <v>0</v>
       </c>
       <c r="U80" t="n">
-        <v>235500</v>
+        <v>239500</v>
       </c>
       <c r="V80" t="n">
         <v>215000</v>
       </c>
       <c r="W80" t="n">
-        <v>9.5</v>
+        <v>11.4</v>
       </c>
     </row>
     <row r="81">
@@ -5157,13 +5157,13 @@
         <v>0</v>
       </c>
       <c r="U81" t="n">
-        <v>2570</v>
+        <v>2590</v>
       </c>
       <c r="V81" t="n">
         <v>2505</v>
       </c>
       <c r="W81" t="n">
-        <v>2.6</v>
+        <v>3.4</v>
       </c>
     </row>
     <row r="82">
@@ -5205,7 +5205,7 @@
         <v>133061.2</v>
       </c>
       <c r="U82" t="n">
-        <v>30700</v>
+        <v>30600</v>
       </c>
     </row>
     <row r="83">
@@ -5247,7 +5247,7 @@
         <v>21395.8</v>
       </c>
       <c r="U83" t="n">
-        <v>88400</v>
+        <v>88800</v>
       </c>
     </row>
     <row r="84">
@@ -5313,13 +5313,13 @@
         <v>0.4</v>
       </c>
       <c r="U84" t="n">
-        <v>87900</v>
+        <v>87700</v>
       </c>
       <c r="V84" t="n">
         <v>89100</v>
       </c>
       <c r="W84" t="n">
-        <v>-1.3</v>
+        <v>-1.6</v>
       </c>
     </row>
     <row r="85">
@@ -5361,7 +5361,7 @@
         <v>2300</v>
       </c>
       <c r="U85" t="n">
-        <v>73900</v>
+        <v>73700</v>
       </c>
     </row>
     <row r="86">
@@ -5427,13 +5427,13 @@
         <v>0</v>
       </c>
       <c r="U86" t="n">
-        <v>20400</v>
+        <v>20450</v>
       </c>
       <c r="V86" t="n">
         <v>21050</v>
       </c>
       <c r="W86" t="n">
-        <v>-3.1</v>
+        <v>-2.9</v>
       </c>
     </row>
     <row r="87">
@@ -5499,13 +5499,13 @@
         <v>0</v>
       </c>
       <c r="U87" t="n">
-        <v>219000</v>
+        <v>218000</v>
       </c>
       <c r="V87" t="n">
         <v>220000</v>
       </c>
       <c r="W87" t="n">
-        <v>-0.5</v>
+        <v>-0.9</v>
       </c>
     </row>
     <row r="88">
@@ -5571,13 +5571,13 @@
         <v>0</v>
       </c>
       <c r="U88" t="n">
-        <v>3320</v>
+        <v>3280</v>
       </c>
       <c r="V88" t="n">
         <v>3450</v>
       </c>
       <c r="W88" t="n">
-        <v>-3.8</v>
+        <v>-4.9</v>
       </c>
     </row>
     <row r="89">
@@ -5619,7 +5619,7 @@
         <v>12775.5</v>
       </c>
       <c r="U89" t="n">
-        <v>99900</v>
+        <v>100700</v>
       </c>
     </row>
     <row r="90">
@@ -5661,7 +5661,7 @@
         <v>1161</v>
       </c>
       <c r="U90" t="n">
-        <v>20250</v>
+        <v>20150</v>
       </c>
     </row>
     <row r="91">
@@ -5727,13 +5727,13 @@
         <v>0</v>
       </c>
       <c r="U91" t="n">
-        <v>27450</v>
+        <v>27650</v>
       </c>
       <c r="V91" t="n">
         <v>26550</v>
       </c>
       <c r="W91" t="n">
-        <v>3.4</v>
+        <v>4.1</v>
       </c>
     </row>
     <row r="92">
@@ -5775,7 +5775,7 @@
         <v>9380.1</v>
       </c>
       <c r="U92" t="n">
-        <v>101900</v>
+        <v>102200</v>
       </c>
     </row>
     <row r="93">
@@ -5817,7 +5817,7 @@
         <v>42377.2</v>
       </c>
       <c r="U93" t="n">
-        <v>20850</v>
+        <v>20800</v>
       </c>
     </row>
     <row r="94">
@@ -5883,13 +5883,13 @@
         <v>-0.2</v>
       </c>
       <c r="U94" t="n">
-        <v>49750</v>
+        <v>49900</v>
       </c>
       <c r="V94" t="n">
         <v>52100</v>
       </c>
       <c r="W94" t="n">
-        <v>-4.5</v>
+        <v>-4.2</v>
       </c>
     </row>
     <row r="95">
@@ -5955,13 +5955,13 @@
         <v>0.4</v>
       </c>
       <c r="U95" t="n">
-        <v>346500</v>
+        <v>345500</v>
       </c>
       <c r="V95" t="n">
         <v>353500</v>
       </c>
       <c r="W95" t="n">
-        <v>-2</v>
+        <v>-2.3</v>
       </c>
     </row>
     <row r="96">
@@ -6027,13 +6027,13 @@
         <v>0</v>
       </c>
       <c r="U96" t="n">
-        <v>5700</v>
+        <v>5690</v>
       </c>
       <c r="V96" t="n">
         <v>5770</v>
       </c>
       <c r="W96" t="n">
-        <v>-1.2</v>
+        <v>-1.4</v>
       </c>
     </row>
     <row r="97">
@@ -6075,7 +6075,7 @@
         <v>8603.299999999999</v>
       </c>
       <c r="U97" t="n">
-        <v>43100</v>
+        <v>43150</v>
       </c>
     </row>
     <row r="98">
@@ -6117,7 +6117,7 @@
         <v>3624.1</v>
       </c>
       <c r="U98" t="n">
-        <v>17770</v>
+        <v>17810</v>
       </c>
     </row>
     <row r="99">
@@ -6231,7 +6231,7 @@
         <v>1930.3</v>
       </c>
       <c r="U100" t="n">
-        <v>170700</v>
+        <v>166900</v>
       </c>
     </row>
     <row r="101">
@@ -6270,13 +6270,13 @@
         <v>-1.4</v>
       </c>
       <c r="U101" t="n">
-        <v>11790</v>
+        <v>11810</v>
       </c>
       <c r="V101" t="n">
         <v>11730</v>
       </c>
       <c r="W101" t="n">
-        <v>0.5</v>
+        <v>0.7</v>
       </c>
     </row>
     <row r="102">
@@ -6342,13 +6342,13 @@
         <v>0.2</v>
       </c>
       <c r="U102" t="n">
-        <v>14810</v>
+        <v>14780</v>
       </c>
       <c r="V102" t="n">
         <v>14190</v>
       </c>
       <c r="W102" t="n">
-        <v>4.4</v>
+        <v>4.2</v>
       </c>
     </row>
     <row r="103">
@@ -6390,7 +6390,7 @@
         <v>45800.4</v>
       </c>
       <c r="U103" t="n">
-        <v>290500</v>
+        <v>293000</v>
       </c>
     </row>
     <row r="104">
@@ -6456,13 +6456,13 @@
         <v>0</v>
       </c>
       <c r="U104" t="n">
-        <v>15950</v>
+        <v>16000</v>
       </c>
       <c r="V104" t="n">
         <v>16640</v>
       </c>
       <c r="W104" t="n">
-        <v>-4.1</v>
+        <v>-3.8</v>
       </c>
     </row>
     <row r="105">
@@ -6528,13 +6528,13 @@
         <v>0.5</v>
       </c>
       <c r="U105" t="n">
-        <v>175400</v>
+        <v>174600</v>
       </c>
       <c r="V105" t="n">
         <v>172800</v>
       </c>
       <c r="W105" t="n">
-        <v>1.5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="106">
@@ -6576,7 +6576,7 @@
         <v>20657.3</v>
       </c>
       <c r="U106" t="n">
-        <v>82000</v>
+        <v>81100</v>
       </c>
     </row>
     <row r="107">
@@ -6684,13 +6684,13 @@
         <v>0</v>
       </c>
       <c r="U108" t="n">
-        <v>9600</v>
+        <v>9670</v>
       </c>
       <c r="V108" t="n">
         <v>9670</v>
       </c>
       <c r="W108" t="n">
-        <v>-0.7</v>
+        <v>0</v>
       </c>
     </row>
     <row r="109">
@@ -6732,7 +6732,7 @@
         <v>131827.2</v>
       </c>
       <c r="U109" t="n">
-        <v>573000</v>
+        <v>576000</v>
       </c>
     </row>
     <row r="110">
@@ -6798,13 +6798,13 @@
         <v>0</v>
       </c>
       <c r="U110" t="n">
-        <v>14390</v>
+        <v>14430</v>
       </c>
       <c r="V110" t="n">
         <v>14420</v>
       </c>
       <c r="W110" t="n">
-        <v>-0.2</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="111">
@@ -6870,13 +6870,13 @@
         <v>1.6</v>
       </c>
       <c r="U111" t="n">
-        <v>199200</v>
+        <v>196300</v>
       </c>
       <c r="V111" t="n">
         <v>197500</v>
       </c>
       <c r="W111" t="n">
-        <v>0.9</v>
+        <v>-0.6</v>
       </c>
     </row>
     <row r="112">
@@ -6942,13 +6942,13 @@
         <v>0.3</v>
       </c>
       <c r="U112" t="n">
-        <v>34300</v>
+        <v>33950</v>
       </c>
       <c r="V112" t="n">
         <v>33600</v>
       </c>
       <c r="W112" t="n">
-        <v>2.1</v>
+        <v>1</v>
       </c>
     </row>
     <row r="113">
@@ -7158,13 +7158,13 @@
         <v>0</v>
       </c>
       <c r="U115" t="n">
-        <v>9390</v>
+        <v>9300</v>
       </c>
       <c r="V115" t="n">
         <v>9110</v>
       </c>
       <c r="W115" t="n">
-        <v>3.1</v>
+        <v>2.1</v>
       </c>
     </row>
     <row r="116">
@@ -7206,7 +7206,7 @@
         <v>24626</v>
       </c>
       <c r="U116" t="n">
-        <v>35300</v>
+        <v>35450</v>
       </c>
     </row>
     <row r="117">
@@ -7272,13 +7272,13 @@
         <v>-0.4</v>
       </c>
       <c r="U117" t="n">
-        <v>215000</v>
+        <v>213500</v>
       </c>
       <c r="V117" t="n">
         <v>209000</v>
       </c>
       <c r="W117" t="n">
-        <v>2.9</v>
+        <v>2.2</v>
       </c>
     </row>
     <row r="118">
@@ -7344,13 +7344,13 @@
         <v>0</v>
       </c>
       <c r="U118" t="n">
-        <v>210000</v>
+        <v>208000</v>
       </c>
       <c r="V118" t="n">
         <v>204500</v>
       </c>
       <c r="W118" t="n">
-        <v>2.7</v>
+        <v>1.7</v>
       </c>
     </row>
     <row r="119">
@@ -7392,7 +7392,7 @@
         <v>2373</v>
       </c>
       <c r="U119" t="n">
-        <v>472500</v>
+        <v>467500</v>
       </c>
     </row>
     <row r="120">
@@ -7506,7 +7506,7 @@
         <v>19670.8</v>
       </c>
       <c r="U121" t="n">
-        <v>255500</v>
+        <v>256500</v>
       </c>
     </row>
     <row r="122">
@@ -7572,13 +7572,13 @@
         <v>0</v>
       </c>
       <c r="U122" t="n">
-        <v>9380</v>
+        <v>9430</v>
       </c>
       <c r="V122" t="n">
         <v>9950</v>
       </c>
       <c r="W122" t="n">
-        <v>-5.7</v>
+        <v>-5.2</v>
       </c>
     </row>
     <row r="123">
@@ -7644,13 +7644,13 @@
         <v>-0.1</v>
       </c>
       <c r="U123" t="n">
-        <v>81400</v>
+        <v>82300</v>
       </c>
       <c r="V123" t="n">
         <v>81600</v>
       </c>
       <c r="W123" t="n">
-        <v>-0.2</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="124">
@@ -7716,13 +7716,13 @@
         <v>0.1</v>
       </c>
       <c r="U124" t="n">
-        <v>80300</v>
+        <v>80500</v>
       </c>
       <c r="V124" t="n">
         <v>83500</v>
       </c>
       <c r="W124" t="n">
-        <v>-3.8</v>
+        <v>-3.6</v>
       </c>
     </row>
     <row r="125">
@@ -7764,7 +7764,7 @@
         <v>6843</v>
       </c>
       <c r="U125" t="n">
-        <v>239000</v>
+        <v>233000</v>
       </c>
     </row>
     <row r="126">
@@ -7803,7 +7803,7 @@
         <v>2273</v>
       </c>
       <c r="U126" t="n">
-        <v>25050</v>
+        <v>24700</v>
       </c>
     </row>
     <row r="127">
@@ -7869,13 +7869,13 @@
         <v>0.2</v>
       </c>
       <c r="U127" t="n">
-        <v>18740</v>
+        <v>18620</v>
       </c>
       <c r="V127" t="n">
         <v>19020</v>
       </c>
       <c r="W127" t="n">
-        <v>-1.5</v>
+        <v>-2.1</v>
       </c>
     </row>
     <row r="128">
@@ -7941,13 +7941,13 @@
         <v>-0.1</v>
       </c>
       <c r="U128" t="n">
-        <v>57700</v>
+        <v>56900</v>
       </c>
       <c r="V128" t="n">
         <v>57100</v>
       </c>
       <c r="W128" t="n">
-        <v>1.1</v>
+        <v>-0.4</v>
       </c>
     </row>
     <row r="129">
@@ -8013,13 +8013,13 @@
         <v>-0.8</v>
       </c>
       <c r="U129" t="n">
-        <v>130100</v>
+        <v>128600</v>
       </c>
       <c r="V129" t="n">
         <v>130200</v>
       </c>
       <c r="W129" t="n">
-        <v>-0.1</v>
+        <v>-1.2</v>
       </c>
     </row>
     <row r="130">
@@ -8085,13 +8085,13 @@
         <v>0</v>
       </c>
       <c r="U130" t="n">
-        <v>21800</v>
+        <v>21850</v>
       </c>
       <c r="V130" t="n">
         <v>21950</v>
       </c>
       <c r="W130" t="n">
-        <v>-0.7</v>
+        <v>-0.5</v>
       </c>
     </row>
     <row r="131">
@@ -8133,7 +8133,7 @@
         <v>2090.2</v>
       </c>
       <c r="U131" t="n">
-        <v>46300</v>
+        <v>46000</v>
       </c>
     </row>
     <row r="132">
@@ -8175,7 +8175,7 @@
         <v>4861.5</v>
       </c>
       <c r="U132" t="n">
-        <v>289250</v>
+        <v>291500</v>
       </c>
     </row>
     <row r="133">
@@ -8217,7 +8217,7 @@
         <v>55616.1</v>
       </c>
       <c r="U133" t="n">
-        <v>259500</v>
+        <v>262000</v>
       </c>
     </row>
     <row r="134">
@@ -8259,7 +8259,7 @@
         <v>1507.4</v>
       </c>
       <c r="U134" t="n">
-        <v>127500</v>
+        <v>125000</v>
       </c>
     </row>
     <row r="135">
@@ -8301,7 +8301,7 @@
         <v>87826.2</v>
       </c>
       <c r="U135" t="n">
-        <v>111100</v>
+        <v>110800</v>
       </c>
     </row>
     <row r="136">
@@ -8343,7 +8343,7 @@
         <v>3109.5</v>
       </c>
       <c r="U136" t="n">
-        <v>72100</v>
+        <v>71000</v>
       </c>
     </row>
     <row r="137">
@@ -8409,13 +8409,13 @@
         <v>0</v>
       </c>
       <c r="U137" t="n">
-        <v>98700</v>
+        <v>96800</v>
       </c>
       <c r="V137" t="n">
         <v>99100</v>
       </c>
       <c r="W137" t="n">
-        <v>-0.4</v>
+        <v>-2.3</v>
       </c>
     </row>
     <row r="138">
@@ -8472,13 +8472,13 @@
         <v>0</v>
       </c>
       <c r="U138" t="n">
-        <v>38850</v>
+        <v>39050</v>
       </c>
       <c r="V138" t="n">
         <v>39950</v>
       </c>
       <c r="W138" t="n">
-        <v>-2.8</v>
+        <v>-2.3</v>
       </c>
     </row>
     <row r="139">
@@ -8520,7 +8520,7 @@
         <v>4380.8</v>
       </c>
       <c r="U139" t="n">
-        <v>203000</v>
+        <v>199900</v>
       </c>
     </row>
     <row r="140">
@@ -8586,13 +8586,13 @@
         <v>0</v>
       </c>
       <c r="U140" t="n">
-        <v>117000</v>
+        <v>116200</v>
       </c>
       <c r="V140" t="n">
         <v>123500</v>
       </c>
       <c r="W140" t="n">
-        <v>-5.3</v>
+        <v>-5.9</v>
       </c>
     </row>
     <row r="141">
@@ -8634,7 +8634,7 @@
         <v>7375.3</v>
       </c>
       <c r="U141" t="n">
-        <v>70600</v>
+        <v>69700</v>
       </c>
     </row>
     <row r="142">
@@ -8676,7 +8676,7 @@
         <v>2073.8</v>
       </c>
       <c r="U142" t="n">
-        <v>275000</v>
+        <v>277500</v>
       </c>
     </row>
     <row r="143">
@@ -8742,13 +8742,13 @@
         <v>0</v>
       </c>
       <c r="U143" t="n">
-        <v>26150</v>
+        <v>27250</v>
       </c>
       <c r="V143" t="n">
         <v>26100</v>
       </c>
       <c r="W143" t="n">
-        <v>0.2</v>
+        <v>4.4</v>
       </c>
     </row>
     <row r="144">
@@ -8814,13 +8814,13 @@
         <v>0</v>
       </c>
       <c r="U144" t="n">
-        <v>215500</v>
+        <v>214500</v>
       </c>
       <c r="V144" t="n">
         <v>198700</v>
       </c>
       <c r="W144" t="n">
-        <v>8.5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="145">
@@ -8886,13 +8886,13 @@
         <v>0</v>
       </c>
       <c r="U145" t="n">
-        <v>113500</v>
+        <v>114500</v>
       </c>
       <c r="V145" t="n">
         <v>110500</v>
       </c>
       <c r="W145" t="n">
-        <v>2.7</v>
+        <v>3.6</v>
       </c>
     </row>
     <row r="146">
@@ -8958,13 +8958,13 @@
         <v>0</v>
       </c>
       <c r="U146" t="n">
-        <v>36450</v>
+        <v>37000</v>
       </c>
       <c r="V146" t="n">
         <v>37000</v>
       </c>
       <c r="W146" t="n">
-        <v>-1.5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="147">
@@ -9006,7 +9006,7 @@
         <v>4756</v>
       </c>
       <c r="U147" t="n">
-        <v>45950</v>
+        <v>45000</v>
       </c>
     </row>
     <row r="148">
@@ -9072,13 +9072,13 @@
         <v>0</v>
       </c>
       <c r="U148" t="n">
-        <v>178600</v>
+        <v>177900</v>
       </c>
       <c r="V148" t="n">
         <v>180100</v>
       </c>
       <c r="W148" t="n">
-        <v>-0.8</v>
+        <v>-1.2</v>
       </c>
     </row>
     <row r="149">
@@ -9120,7 +9120,7 @@
         <v>1060</v>
       </c>
       <c r="U149" t="n">
-        <v>16330</v>
+        <v>16360</v>
       </c>
     </row>
     <row r="150">
@@ -9234,7 +9234,7 @@
         <v>5553.6</v>
       </c>
       <c r="U151" t="n">
-        <v>92700</v>
+        <v>91200</v>
       </c>
     </row>
     <row r="152">
@@ -9276,7 +9276,7 @@
         <v>33383.2</v>
       </c>
       <c r="U152" t="n">
-        <v>182300</v>
+        <v>181700</v>
       </c>
     </row>
     <row r="153">
@@ -9318,7 +9318,7 @@
         <v>4094</v>
       </c>
       <c r="U153" t="n">
-        <v>78700</v>
+        <v>78800</v>
       </c>
     </row>
     <row r="154">
@@ -9384,13 +9384,13 @@
         <v>0</v>
       </c>
       <c r="U154" t="n">
-        <v>48900</v>
+        <v>48950</v>
       </c>
       <c r="V154" t="n">
         <v>52100</v>
       </c>
       <c r="W154" t="n">
-        <v>-6.1</v>
+        <v>-6</v>
       </c>
     </row>
     <row r="155">
@@ -9456,13 +9456,13 @@
         <v>0</v>
       </c>
       <c r="U155" t="n">
-        <v>6900</v>
+        <v>6810</v>
       </c>
       <c r="V155" t="n">
         <v>7040</v>
       </c>
       <c r="W155" t="n">
-        <v>-2</v>
+        <v>-3.3</v>
       </c>
     </row>
     <row r="156">
@@ -9501,13 +9501,13 @@
         <v>0</v>
       </c>
       <c r="U156" t="n">
-        <v>9970</v>
+        <v>9990</v>
       </c>
       <c r="V156" t="n">
         <v>10350</v>
       </c>
       <c r="W156" t="n">
-        <v>-3.7</v>
+        <v>-3.5</v>
       </c>
     </row>
     <row r="157">
@@ -9546,13 +9546,13 @@
         <v>0</v>
       </c>
       <c r="U157" t="n">
-        <v>13050</v>
+        <v>12700</v>
       </c>
       <c r="V157" t="n">
         <v>11550</v>
       </c>
       <c r="W157" t="n">
-        <v>13</v>
+        <v>10</v>
       </c>
     </row>
     <row r="158">
@@ -9666,7 +9666,7 @@
         <v>36994</v>
       </c>
       <c r="U159" t="n">
-        <v>112000</v>
+        <v>114300</v>
       </c>
     </row>
     <row r="160">
@@ -9732,13 +9732,13 @@
         <v>-0.4</v>
       </c>
       <c r="U160" t="n">
-        <v>691000</v>
+        <v>690000</v>
       </c>
       <c r="V160" t="n">
         <v>737000</v>
       </c>
       <c r="W160" t="n">
-        <v>-6.2</v>
+        <v>-6.4</v>
       </c>
     </row>
     <row r="161">
@@ -9777,13 +9777,13 @@
         <v>0</v>
       </c>
       <c r="U161" t="n">
-        <v>8450</v>
+        <v>8470</v>
       </c>
       <c r="V161" t="n">
         <v>8990</v>
       </c>
       <c r="W161" t="n">
-        <v>-6</v>
+        <v>-5.8</v>
       </c>
     </row>
     <row r="162">
@@ -9825,7 +9825,7 @@
         <v>6392</v>
       </c>
       <c r="U162" t="n">
-        <v>38250</v>
+        <v>38200</v>
       </c>
     </row>
     <row r="163">
@@ -9891,13 +9891,13 @@
         <v>0</v>
       </c>
       <c r="U163" t="n">
-        <v>48000</v>
+        <v>47550</v>
       </c>
       <c r="V163" t="n">
         <v>51600</v>
       </c>
       <c r="W163" t="n">
-        <v>-7</v>
+        <v>-7.8</v>
       </c>
     </row>
     <row r="164">
@@ -9939,7 +9939,7 @@
         <v>2224</v>
       </c>
       <c r="U164" t="n">
-        <v>60400</v>
+        <v>60100</v>
       </c>
     </row>
     <row r="165">
@@ -9981,7 +9981,7 @@
         <v>1800</v>
       </c>
       <c r="U165" t="n">
-        <v>155900</v>
+        <v>154100</v>
       </c>
     </row>
     <row r="166">
@@ -10047,13 +10047,13 @@
         <v>0</v>
       </c>
       <c r="U166" t="n">
-        <v>201000</v>
+        <v>198100</v>
       </c>
       <c r="V166" t="n">
         <v>204000</v>
       </c>
       <c r="W166" t="n">
-        <v>-1.5</v>
+        <v>-2.9</v>
       </c>
     </row>
     <row r="167">
@@ -10137,7 +10137,7 @@
         <v>10708.8</v>
       </c>
       <c r="U168" t="n">
-        <v>5780</v>
+        <v>5820</v>
       </c>
     </row>
     <row r="169">
@@ -10203,13 +10203,13 @@
         <v>0</v>
       </c>
       <c r="U169" t="n">
-        <v>49250</v>
+        <v>49550</v>
       </c>
       <c r="V169" t="n">
         <v>49000</v>
       </c>
       <c r="W169" t="n">
-        <v>0.5</v>
+        <v>1.1</v>
       </c>
     </row>
     <row r="170">
@@ -10275,13 +10275,13 @@
         <v>0</v>
       </c>
       <c r="U170" t="n">
-        <v>60600</v>
+        <v>59800</v>
       </c>
       <c r="V170" t="n">
         <v>55100</v>
       </c>
       <c r="W170" t="n">
-        <v>10</v>
+        <v>8.5</v>
       </c>
     </row>
     <row r="171">
@@ -10347,13 +10347,13 @@
         <v>0</v>
       </c>
       <c r="U171" t="n">
-        <v>142800</v>
+        <v>141900</v>
       </c>
       <c r="V171" t="n">
         <v>142700</v>
       </c>
       <c r="W171" t="n">
-        <v>0.1</v>
+        <v>-0.6</v>
       </c>
     </row>
     <row r="172">
@@ -10386,7 +10386,7 @@
         <v>243</v>
       </c>
       <c r="U172" t="n">
-        <v>13960</v>
+        <v>13980</v>
       </c>
     </row>
     <row r="173">
@@ -10428,7 +10428,7 @@
         <v>1766.5</v>
       </c>
       <c r="U173" t="n">
-        <v>204000</v>
+        <v>203500</v>
       </c>
     </row>
     <row r="174">
@@ -10470,7 +10470,7 @@
         <v>1928.5</v>
       </c>
       <c r="U174" t="n">
-        <v>163400</v>
+        <v>161900</v>
       </c>
     </row>
     <row r="175">
@@ -10536,13 +10536,13 @@
         <v>-2.1</v>
       </c>
       <c r="U175" t="n">
-        <v>17860</v>
+        <v>17840</v>
       </c>
       <c r="V175" t="n">
         <v>17800</v>
       </c>
       <c r="W175" t="n">
-        <v>0.3</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="176">
@@ -10608,13 +10608,13 @@
         <v>0</v>
       </c>
       <c r="U176" t="n">
-        <v>34500</v>
+        <v>34100</v>
       </c>
       <c r="V176" t="n">
         <v>33900</v>
       </c>
       <c r="W176" t="n">
-        <v>1.8</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="177">
@@ -10656,7 +10656,7 @@
         <v>43017.9</v>
       </c>
       <c r="U177" t="n">
-        <v>157700</v>
+        <v>158900</v>
       </c>
     </row>
     <row r="178">
@@ -10722,13 +10722,13 @@
         <v>0</v>
       </c>
       <c r="U178" t="n">
-        <v>178600</v>
+        <v>178800</v>
       </c>
       <c r="V178" t="n">
         <v>175000</v>
       </c>
       <c r="W178" t="n">
-        <v>2.1</v>
+        <v>2.2</v>
       </c>
     </row>
     <row r="179">
@@ -10761,7 +10761,7 @@
         <v>156</v>
       </c>
       <c r="U179" t="n">
-        <v>29150</v>
+        <v>28850</v>
       </c>
     </row>
     <row r="180">
@@ -10827,7 +10827,7 @@
         <v>0</v>
       </c>
       <c r="U180" t="n">
-        <v>15960</v>
+        <v>15950</v>
       </c>
       <c r="V180" t="n">
         <v>16200</v>
@@ -10899,13 +10899,13 @@
         <v>0</v>
       </c>
       <c r="U181" t="n">
-        <v>80000</v>
+        <v>80300</v>
       </c>
       <c r="V181" t="n">
         <v>78900</v>
       </c>
       <c r="W181" t="n">
-        <v>1.4</v>
+        <v>1.8</v>
       </c>
     </row>
     <row r="182">
@@ -10971,13 +10971,13 @@
         <v>0</v>
       </c>
       <c r="U182" t="n">
-        <v>78200</v>
+        <v>77900</v>
       </c>
       <c r="V182" t="n">
         <v>79700</v>
       </c>
       <c r="W182" t="n">
-        <v>-1.9</v>
+        <v>-2.3</v>
       </c>
     </row>
     <row r="183">
@@ -11019,7 +11019,7 @@
         <v>98431.89999999999</v>
       </c>
       <c r="U183" t="n">
-        <v>174000</v>
+        <v>173800</v>
       </c>
     </row>
     <row r="184">
@@ -11085,13 +11085,13 @@
         <v>0</v>
       </c>
       <c r="U184" t="n">
-        <v>292000</v>
+        <v>283500</v>
       </c>
       <c r="V184" t="n">
         <v>307500</v>
       </c>
       <c r="W184" t="n">
-        <v>-5</v>
+        <v>-7.8</v>
       </c>
     </row>
     <row r="185">
@@ -11133,7 +11133,7 @@
         <v>7986.8</v>
       </c>
       <c r="U185" t="n">
-        <v>71400</v>
+        <v>71100</v>
       </c>
     </row>
     <row r="186">
@@ -11175,7 +11175,7 @@
         <v>2642.8</v>
       </c>
       <c r="U186" t="n">
-        <v>50900</v>
+        <v>52800</v>
       </c>
     </row>
     <row r="187">
@@ -11262,7 +11262,7 @@
         <v>3361.8</v>
       </c>
       <c r="U188" t="n">
-        <v>55600</v>
+        <v>55700</v>
       </c>
     </row>
     <row r="189">
@@ -11328,13 +11328,13 @@
         <v>0</v>
       </c>
       <c r="U189" t="n">
-        <v>42600</v>
+        <v>42700</v>
       </c>
       <c r="V189" t="n">
         <v>43600</v>
       </c>
       <c r="W189" t="n">
-        <v>-2.3</v>
+        <v>-2.1</v>
       </c>
     </row>
     <row r="190">
@@ -11400,13 +11400,13 @@
         <v>0</v>
       </c>
       <c r="U190" t="n">
-        <v>505000</v>
+        <v>503000</v>
       </c>
       <c r="V190" t="n">
         <v>505000</v>
       </c>
       <c r="W190" t="n">
-        <v>0</v>
+        <v>-0.4</v>
       </c>
     </row>
     <row r="191">
@@ -11448,7 +11448,7 @@
         <v>3054</v>
       </c>
       <c r="U191" t="n">
-        <v>287500</v>
+        <v>293000</v>
       </c>
     </row>
     <row r="192">
@@ -11490,7 +11490,7 @@
         <v>35646.6</v>
       </c>
       <c r="U192" t="n">
-        <v>130300</v>
+        <v>132500</v>
       </c>
     </row>
     <row r="193">
@@ -11532,7 +11532,7 @@
         <v>11736.9</v>
       </c>
       <c r="U193" t="n">
-        <v>16410</v>
+        <v>16470</v>
       </c>
     </row>
     <row r="194">
@@ -11574,7 +11574,7 @@
         <v>7286.1</v>
       </c>
       <c r="U194" t="n">
-        <v>18810</v>
+        <v>18700</v>
       </c>
     </row>
     <row r="195">
@@ -11616,7 +11616,7 @@
         <v>6040.5</v>
       </c>
       <c r="U195" t="n">
-        <v>71900</v>
+        <v>72000</v>
       </c>
     </row>
     <row r="196">
@@ -11658,7 +11658,7 @@
         <v>842.6</v>
       </c>
       <c r="U196" t="n">
-        <v>261500</v>
+        <v>263500</v>
       </c>
     </row>
     <row r="197">
@@ -11715,13 +11715,13 @@
         <v>0</v>
       </c>
       <c r="U197" t="n">
-        <v>80900</v>
+        <v>79400</v>
       </c>
       <c r="V197" t="n">
         <v>81900</v>
       </c>
       <c r="W197" t="n">
-        <v>-1.2</v>
+        <v>-3.1</v>
       </c>
     </row>
     <row r="198">
@@ -11787,13 +11787,13 @@
         <v>-2.3</v>
       </c>
       <c r="U198" t="n">
-        <v>188900</v>
+        <v>185700</v>
       </c>
       <c r="V198" t="n">
         <v>215000</v>
       </c>
       <c r="W198" t="n">
-        <v>-12.1</v>
+        <v>-13.6</v>
       </c>
     </row>
     <row r="199">
@@ -11904,13 +11904,13 @@
         <v>0</v>
       </c>
       <c r="U200" t="n">
-        <v>10500</v>
+        <v>10400</v>
       </c>
       <c r="V200" t="n">
         <v>10050</v>
       </c>
       <c r="W200" t="n">
-        <v>4.5</v>
+        <v>3.5</v>
       </c>
     </row>
     <row r="201">
@@ -11976,13 +11976,13 @@
         <v>0</v>
       </c>
       <c r="U201" t="n">
-        <v>58400</v>
+        <v>59300</v>
       </c>
       <c r="V201" t="n">
         <v>60700</v>
       </c>
       <c r="W201" t="n">
-        <v>-3.8</v>
+        <v>-2.3</v>
       </c>
     </row>
     <row r="202">
@@ -12048,13 +12048,13 @@
         <v>0</v>
       </c>
       <c r="U202" t="n">
-        <v>147800</v>
+        <v>148000</v>
       </c>
       <c r="V202" t="n">
         <v>145500</v>
       </c>
       <c r="W202" t="n">
-        <v>1.6</v>
+        <v>1.7</v>
       </c>
     </row>
     <row r="203">
@@ -12120,13 +12120,13 @@
         <v>0</v>
       </c>
       <c r="U203" t="n">
-        <v>34650</v>
+        <v>34750</v>
       </c>
       <c r="V203" t="n">
         <v>35700</v>
       </c>
       <c r="W203" t="n">
-        <v>-2.9</v>
+        <v>-2.7</v>
       </c>
     </row>
     <row r="204">
@@ -12210,7 +12210,7 @@
         <v>3491.5</v>
       </c>
       <c r="U205" t="n">
-        <v>36150</v>
+        <v>36300</v>
       </c>
     </row>
     <row r="206">
@@ -12276,13 +12276,13 @@
         <v>0</v>
       </c>
       <c r="U206" t="n">
-        <v>64800</v>
+        <v>65200</v>
       </c>
       <c r="V206" t="n">
         <v>64400</v>
       </c>
       <c r="W206" t="n">
-        <v>0.6</v>
+        <v>1.2</v>
       </c>
     </row>
     <row r="207">
@@ -12348,13 +12348,13 @@
         <v>0</v>
       </c>
       <c r="U207" t="n">
-        <v>68400</v>
+        <v>67200</v>
       </c>
       <c r="V207" t="n">
         <v>68600</v>
       </c>
       <c r="W207" t="n">
-        <v>-0.3</v>
+        <v>-2</v>
       </c>
     </row>
     <row r="208">
@@ -12420,13 +12420,13 @@
         <v>0</v>
       </c>
       <c r="U208" t="n">
-        <v>59000</v>
+        <v>58600</v>
       </c>
       <c r="V208" t="n">
         <v>59000</v>
       </c>
       <c r="W208" t="n">
-        <v>0</v>
+        <v>-0.7</v>
       </c>
     </row>
     <row r="209">
@@ -12492,13 +12492,13 @@
         <v>0</v>
       </c>
       <c r="U209" t="n">
-        <v>272500</v>
+        <v>269500</v>
       </c>
       <c r="V209" t="n">
         <v>274000</v>
       </c>
       <c r="W209" t="n">
-        <v>-0.5</v>
+        <v>-1.6</v>
       </c>
     </row>
     <row r="210">
@@ -12564,13 +12564,13 @@
         <v>0</v>
       </c>
       <c r="U210" t="n">
-        <v>39250</v>
+        <v>39150</v>
       </c>
       <c r="V210" t="n">
         <v>38900</v>
       </c>
       <c r="W210" t="n">
-        <v>0.9</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="211">
@@ -12612,7 +12612,7 @@
         <v>5785</v>
       </c>
       <c r="U211" t="n">
-        <v>254000</v>
+        <v>251000</v>
       </c>
     </row>
     <row r="212">
@@ -12678,13 +12678,13 @@
         <v>0</v>
       </c>
       <c r="U212" t="n">
-        <v>46450</v>
+        <v>46250</v>
       </c>
       <c r="V212" t="n">
         <v>48250</v>
       </c>
       <c r="W212" t="n">
-        <v>-3.7</v>
+        <v>-4.1</v>
       </c>
     </row>
     <row r="213">
@@ -12750,13 +12750,13 @@
         <v>0</v>
       </c>
       <c r="U213" t="n">
-        <v>1388000</v>
+        <v>1390000</v>
       </c>
       <c r="V213" t="n">
         <v>1399000</v>
       </c>
       <c r="W213" t="n">
-        <v>-0.8</v>
+        <v>-0.6</v>
       </c>
     </row>
     <row r="214">
@@ -12822,13 +12822,13 @@
         <v>-1.2</v>
       </c>
       <c r="U214" t="n">
-        <v>31000</v>
+        <v>30850</v>
       </c>
       <c r="V214" t="n">
         <v>31450</v>
       </c>
       <c r="W214" t="n">
-        <v>-1.4</v>
+        <v>-1.9</v>
       </c>
     </row>
     <row r="215">
@@ -12894,13 +12894,13 @@
         <v>0.7</v>
       </c>
       <c r="U215" t="n">
-        <v>321000</v>
+        <v>319000</v>
       </c>
       <c r="V215" t="n">
         <v>327000</v>
       </c>
       <c r="W215" t="n">
-        <v>-1.8</v>
+        <v>-2.4</v>
       </c>
     </row>
     <row r="216">
@@ -12966,13 +12966,13 @@
         <v>0</v>
       </c>
       <c r="U216" t="n">
-        <v>57200</v>
+        <v>56400</v>
       </c>
       <c r="V216" t="n">
         <v>61300</v>
       </c>
       <c r="W216" t="n">
-        <v>-6.7</v>
+        <v>-8</v>
       </c>
     </row>
     <row r="217">
@@ -13014,7 +13014,7 @@
         <v>5480.8</v>
       </c>
       <c r="U217" t="n">
-        <v>149300</v>
+        <v>145100</v>
       </c>
     </row>
     <row r="218">
@@ -13080,13 +13080,13 @@
         <v>0</v>
       </c>
       <c r="U218" t="n">
-        <v>93300</v>
+        <v>92800</v>
       </c>
       <c r="V218" t="n">
         <v>92700</v>
       </c>
       <c r="W218" t="n">
-        <v>0.6</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="219">
@@ -13128,7 +13128,7 @@
         <v>3478.3</v>
       </c>
       <c r="U219" t="n">
-        <v>126600</v>
+        <v>123700</v>
       </c>
     </row>
     <row r="220">
@@ -13194,13 +13194,13 @@
         <v>0</v>
       </c>
       <c r="U220" t="n">
-        <v>58100</v>
+        <v>58300</v>
       </c>
       <c r="V220" t="n">
         <v>59400</v>
       </c>
       <c r="W220" t="n">
-        <v>-2.2</v>
+        <v>-1.9</v>
       </c>
     </row>
     <row r="221">
@@ -13266,13 +13266,13 @@
         <v>0</v>
       </c>
       <c r="U221" t="n">
-        <v>126600</v>
+        <v>125000</v>
       </c>
       <c r="V221" t="n">
         <v>132100</v>
       </c>
       <c r="W221" t="n">
-        <v>-4.2</v>
+        <v>-5.4</v>
       </c>
     </row>
     <row r="222">
@@ -13338,13 +13338,13 @@
         <v>0</v>
       </c>
       <c r="U222" t="n">
-        <v>107500</v>
+        <v>110500</v>
       </c>
       <c r="V222" t="n">
         <v>105300</v>
       </c>
       <c r="W222" t="n">
-        <v>2.1</v>
+        <v>4.9</v>
       </c>
     </row>
     <row r="223">
@@ -13410,13 +13410,13 @@
         <v>0</v>
       </c>
       <c r="U223" t="n">
-        <v>35150</v>
+        <v>35300</v>
       </c>
       <c r="V223" t="n">
         <v>34750</v>
       </c>
       <c r="W223" t="n">
-        <v>1.2</v>
+        <v>1.6</v>
       </c>
     </row>
     <row r="224">
@@ -13482,13 +13482,13 @@
         <v>0</v>
       </c>
       <c r="U224" t="n">
-        <v>62300</v>
+        <v>62100</v>
       </c>
       <c r="V224" t="n">
         <v>61700</v>
       </c>
       <c r="W224" t="n">
-        <v>1</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="225">
@@ -13602,7 +13602,7 @@
         <v>4611.6</v>
       </c>
       <c r="U226" t="n">
-        <v>38900</v>
+        <v>38700</v>
       </c>
     </row>
     <row r="227">
@@ -13668,13 +13668,13 @@
         <v>0</v>
       </c>
       <c r="U227" t="n">
-        <v>201000</v>
+        <v>200500</v>
       </c>
       <c r="V227" t="n">
         <v>204500</v>
       </c>
       <c r="W227" t="n">
-        <v>-1.7</v>
+        <v>-2</v>
       </c>
     </row>
     <row r="228">
@@ -13716,7 +13716,7 @@
         <v>2262.8</v>
       </c>
       <c r="U228" t="n">
-        <v>33500</v>
+        <v>33100</v>
       </c>
     </row>
     <row r="229">
@@ -13758,7 +13758,7 @@
         <v>132859.2</v>
       </c>
       <c r="U229" t="n">
-        <v>210500</v>
+        <v>210000</v>
       </c>
     </row>
     <row r="230">
@@ -13896,13 +13896,13 @@
         <v>0</v>
       </c>
       <c r="U231" t="n">
-        <v>129900</v>
+        <v>128400</v>
       </c>
       <c r="V231" t="n">
         <v>140400</v>
       </c>
       <c r="W231" t="n">
-        <v>-7.5</v>
+        <v>-8.5</v>
       </c>
     </row>
     <row r="232">
@@ -13968,13 +13968,13 @@
         <v>0</v>
       </c>
       <c r="U232" t="n">
-        <v>111300</v>
+        <v>111600</v>
       </c>
       <c r="V232" t="n">
         <v>112500</v>
       </c>
       <c r="W232" t="n">
-        <v>-1.1</v>
+        <v>-0.8</v>
       </c>
     </row>
     <row r="233">
@@ -14040,13 +14040,13 @@
         <v>0</v>
       </c>
       <c r="U233" t="n">
-        <v>72800</v>
+        <v>72600</v>
       </c>
       <c r="V233" t="n">
         <v>79900</v>
       </c>
       <c r="W233" t="n">
-        <v>-8.9</v>
+        <v>-9.1</v>
       </c>
     </row>
     <row r="234">
@@ -14112,13 +14112,13 @@
         <v>0</v>
       </c>
       <c r="U234" t="n">
-        <v>6020</v>
+        <v>5960</v>
       </c>
       <c r="V234" t="n">
         <v>5820</v>
       </c>
       <c r="W234" t="n">
-        <v>3.4</v>
+        <v>2.4</v>
       </c>
     </row>
     <row r="235">
@@ -14175,13 +14175,13 @@
         <v>0</v>
       </c>
       <c r="U235" t="n">
-        <v>426000</v>
+        <v>422500</v>
       </c>
       <c r="V235" t="n">
         <v>434500</v>
       </c>
       <c r="W235" t="n">
-        <v>-2</v>
+        <v>-2.8</v>
       </c>
     </row>
     <row r="236">
@@ -14247,13 +14247,13 @@
         <v>0</v>
       </c>
       <c r="U236" t="n">
-        <v>366000</v>
+        <v>367000</v>
       </c>
       <c r="V236" t="n">
         <v>368000</v>
       </c>
       <c r="W236" t="n">
-        <v>-0.5</v>
+        <v>-0.3</v>
       </c>
     </row>
     <row r="237">
@@ -14319,7 +14319,7 @@
         <v>0</v>
       </c>
       <c r="U237" t="n">
-        <v>126000</v>
+        <v>125900</v>
       </c>
       <c r="V237" t="n">
         <v>127100</v>
@@ -14367,7 +14367,7 @@
         <v>3671.2</v>
       </c>
       <c r="U238" t="n">
-        <v>133000</v>
+        <v>133500</v>
       </c>
     </row>
     <row r="239">
@@ -14409,7 +14409,7 @@
         <v>2230</v>
       </c>
       <c r="U239" t="n">
-        <v>51600</v>
+        <v>51700</v>
       </c>
     </row>
     <row r="240">
@@ -14523,7 +14523,7 @@
         <v>6487.3</v>
       </c>
       <c r="U241" t="n">
-        <v>313500</v>
+        <v>311000</v>
       </c>
     </row>
     <row r="242">
@@ -14589,13 +14589,13 @@
         <v>0.3</v>
       </c>
       <c r="U242" t="n">
-        <v>2787000</v>
+        <v>2784000</v>
       </c>
       <c r="V242" t="n">
         <v>2888000</v>
       </c>
       <c r="W242" t="n">
-        <v>-3.5</v>
+        <v>-3.6</v>
       </c>
     </row>
     <row r="243">
@@ -14637,7 +14637,7 @@
         <v>2979.5</v>
       </c>
       <c r="U243" t="n">
-        <v>165100</v>
+        <v>165900</v>
       </c>
     </row>
     <row r="244">
@@ -14679,7 +14679,7 @@
         <v>1723.5</v>
       </c>
       <c r="U244" t="n">
-        <v>16330</v>
+        <v>16280</v>
       </c>
     </row>
     <row r="245">
@@ -14736,13 +14736,13 @@
         <v>0</v>
       </c>
       <c r="U245" t="n">
-        <v>36350</v>
+        <v>36100</v>
       </c>
       <c r="V245" t="n">
         <v>35350</v>
       </c>
       <c r="W245" t="n">
-        <v>2.8</v>
+        <v>2.1</v>
       </c>
     </row>
     <row r="246">
@@ -14808,13 +14808,13 @@
         <v>4.6</v>
       </c>
       <c r="U246" t="n">
-        <v>145800</v>
+        <v>146200</v>
       </c>
       <c r="V246" t="n">
         <v>148000</v>
       </c>
       <c r="W246" t="n">
-        <v>-1.5</v>
+        <v>-1.2</v>
       </c>
     </row>
     <row r="247">
@@ -14856,7 +14856,7 @@
         <v>4543.1</v>
       </c>
       <c r="U247" t="n">
-        <v>378000</v>
+        <v>374500</v>
       </c>
     </row>
     <row r="248">
@@ -14898,7 +14898,7 @@
         <v>50413.7</v>
       </c>
       <c r="U248" t="n">
-        <v>36250</v>
+        <v>36200</v>
       </c>
     </row>
     <row r="249">
@@ -14964,13 +14964,13 @@
         <v>0</v>
       </c>
       <c r="U249" t="n">
-        <v>9870</v>
+        <v>9680</v>
       </c>
       <c r="V249" t="n">
         <v>10040</v>
       </c>
       <c r="W249" t="n">
-        <v>-1.7</v>
+        <v>-3.6</v>
       </c>
     </row>
     <row r="250">
@@ -15012,7 +15012,7 @@
         <v>2609.8</v>
       </c>
       <c r="U250" t="n">
-        <v>142700</v>
+        <v>141000</v>
       </c>
     </row>
     <row r="251">
@@ -15078,13 +15078,13 @@
         <v>0</v>
       </c>
       <c r="U251" t="n">
-        <v>20350</v>
+        <v>20400</v>
       </c>
       <c r="V251" t="n">
         <v>20550</v>
       </c>
       <c r="W251" t="n">
-        <v>-1</v>
+        <v>-0.7</v>
       </c>
     </row>
     <row r="252">
@@ -15150,13 +15150,13 @@
         <v>0</v>
       </c>
       <c r="U252" t="n">
-        <v>76300</v>
+        <v>76000</v>
       </c>
       <c r="V252" t="n">
         <v>77900</v>
       </c>
       <c r="W252" t="n">
-        <v>-2.1</v>
+        <v>-2.4</v>
       </c>
     </row>
     <row r="253">
@@ -15222,13 +15222,13 @@
         <v>0</v>
       </c>
       <c r="U253" t="n">
-        <v>441250</v>
+        <v>439000</v>
       </c>
       <c r="V253" t="n">
         <v>462000</v>
       </c>
       <c r="W253" t="n">
-        <v>-4.5</v>
+        <v>-5</v>
       </c>
     </row>
     <row r="254">
@@ -15294,13 +15294,13 @@
         <v>-0.1</v>
       </c>
       <c r="U254" t="n">
-        <v>162500</v>
+        <v>161900</v>
       </c>
       <c r="V254" t="n">
         <v>166700</v>
       </c>
       <c r="W254" t="n">
-        <v>-2.5</v>
+        <v>-2.9</v>
       </c>
     </row>
     <row r="255">
@@ -15366,13 +15366,13 @@
         <v>0</v>
       </c>
       <c r="U255" t="n">
-        <v>123000</v>
+        <v>121700</v>
       </c>
       <c r="V255" t="n">
         <v>103100</v>
       </c>
       <c r="W255" t="n">
-        <v>19.3</v>
+        <v>18</v>
       </c>
     </row>
     <row r="256">
@@ -15414,7 +15414,7 @@
         <v>3590.6</v>
       </c>
       <c r="U256" t="n">
-        <v>373500</v>
+        <v>364500</v>
       </c>
     </row>
     <row r="257">
@@ -15456,7 +15456,7 @@
         <v>-130.5</v>
       </c>
       <c r="U257" t="n">
-        <v>18150</v>
+        <v>18280</v>
       </c>
     </row>
     <row r="258">
@@ -15522,13 +15522,13 @@
         <v>-0.4</v>
       </c>
       <c r="U258" t="n">
-        <v>360000</v>
+        <v>360500</v>
       </c>
       <c r="V258" t="n">
         <v>363500</v>
       </c>
       <c r="W258" t="n">
-        <v>-1</v>
+        <v>-0.8</v>
       </c>
     </row>
     <row r="259">
@@ -15666,13 +15666,13 @@
         <v>0</v>
       </c>
       <c r="U260" t="n">
-        <v>16960</v>
+        <v>17060</v>
       </c>
       <c r="V260" t="n">
         <v>17140</v>
       </c>
       <c r="W260" t="n">
-        <v>-1.1</v>
+        <v>-0.5</v>
       </c>
     </row>
     <row r="261">
@@ -15714,7 +15714,7 @@
         <v>2468.7</v>
       </c>
       <c r="U261" t="n">
-        <v>41250</v>
+        <v>40900</v>
       </c>
     </row>
     <row r="262">
@@ -15756,7 +15756,7 @@
         <v>6274.3</v>
       </c>
       <c r="U262" t="n">
-        <v>69300</v>
+        <v>69100</v>
       </c>
     </row>
     <row r="263">
@@ -15795,13 +15795,13 @@
         <v>0</v>
       </c>
       <c r="U263" t="n">
-        <v>42700</v>
+        <v>41850</v>
       </c>
       <c r="V263" t="n">
         <v>40850</v>
       </c>
       <c r="W263" t="n">
-        <v>4.5</v>
+        <v>2.4</v>
       </c>
     </row>
     <row r="264">
@@ -15840,13 +15840,13 @@
         <v>0</v>
       </c>
       <c r="U264" t="n">
-        <v>31900</v>
+        <v>31450</v>
       </c>
       <c r="V264" t="n">
         <v>28900</v>
       </c>
       <c r="W264" t="n">
-        <v>10.4</v>
+        <v>8.800000000000001</v>
       </c>
     </row>
     <row r="265">
@@ -15888,7 +15888,7 @@
         <v>607606</v>
       </c>
       <c r="U265" t="n">
-        <v>1104000</v>
+        <v>1092000</v>
       </c>
     </row>
     <row r="266">
@@ -15921,7 +15921,7 @@
         <v>298</v>
       </c>
       <c r="U266" t="n">
-        <v>55800</v>
+        <v>55400</v>
       </c>
     </row>
     <row r="267">
@@ -15987,13 +15987,13 @@
         <v>0</v>
       </c>
       <c r="U267" t="n">
-        <v>123700</v>
+        <v>125900</v>
       </c>
       <c r="V267" t="n">
         <v>112100</v>
       </c>
       <c r="W267" t="n">
-        <v>10.3</v>
+        <v>12.3</v>
       </c>
     </row>
     <row r="268">
@@ -16107,7 +16107,7 @@
         <v>3103</v>
       </c>
       <c r="U269" t="n">
-        <v>82000</v>
+        <v>80000</v>
       </c>
     </row>
     <row r="270">
@@ -16173,13 +16173,13 @@
         <v>0</v>
       </c>
       <c r="U270" t="n">
-        <v>242000</v>
+        <v>242500</v>
       </c>
       <c r="V270" t="n">
         <v>244000</v>
       </c>
       <c r="W270" t="n">
-        <v>-0.8</v>
+        <v>-0.6</v>
       </c>
     </row>
     <row r="271">
@@ -16221,7 +16221,7 @@
         <v>1966.7</v>
       </c>
       <c r="U271" t="n">
-        <v>80700</v>
+        <v>79600</v>
       </c>
     </row>
     <row r="272">
@@ -16320,13 +16320,13 @@
         <v>0</v>
       </c>
       <c r="U273" t="n">
-        <v>9470</v>
+        <v>9400</v>
       </c>
       <c r="V273" t="n">
         <v>10260</v>
       </c>
       <c r="W273" t="n">
-        <v>-7.7</v>
+        <v>-8.4</v>
       </c>
     </row>
     <row r="274">
@@ -16464,13 +16464,13 @@
         <v>-0.5</v>
       </c>
       <c r="U275" t="n">
-        <v>181400</v>
+        <v>183100</v>
       </c>
       <c r="V275" t="n">
         <v>182100</v>
       </c>
       <c r="W275" t="n">
-        <v>-0.4</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="276">
@@ -16536,13 +16536,13 @@
         <v>0</v>
       </c>
       <c r="U276" t="n">
-        <v>17980</v>
+        <v>18120</v>
       </c>
       <c r="V276" t="n">
         <v>18730</v>
       </c>
       <c r="W276" t="n">
-        <v>-4</v>
+        <v>-3.3</v>
       </c>
     </row>
     <row r="277">
@@ -16608,13 +16608,13 @@
         <v>0</v>
       </c>
       <c r="U277" t="n">
-        <v>46600</v>
+        <v>46100</v>
       </c>
       <c r="V277" t="n">
         <v>47350</v>
       </c>
       <c r="W277" t="n">
-        <v>-1.6</v>
+        <v>-2.6</v>
       </c>
     </row>
     <row r="278">
@@ -16653,13 +16653,13 @@
         <v>0</v>
       </c>
       <c r="U278" t="n">
-        <v>30550</v>
+        <v>29700</v>
       </c>
       <c r="V278" t="n">
         <v>29950</v>
       </c>
       <c r="W278" t="n">
-        <v>2</v>
+        <v>-0.8</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore(consensus): 주간 컨센 스냅샷 2026-10-24
</commit_message>
<xml_diff>
--- a/telegram_research_dashboard/static/consensus_full.xlsx
+++ b/telegram_research_dashboard/static/consensus_full.xlsx
@@ -465,7 +465,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>영업이익 컨센(KOSPI200·KOSDAQ50·커버리지) · 기준일 2026-10-23 · 전주 2026-10-17</t>
+          <t>영업이익 컨센(KOSPI200·KOSDAQ50·커버리지) · 기준일 2026-10-24 · 전주 2026-10-17</t>
         </is>
       </c>
     </row>
@@ -1058,70 +1058,70 @@
         </is>
       </c>
       <c r="F7" t="n">
-        <v>1904</v>
+        <v>1928</v>
       </c>
       <c r="G7" t="n">
-        <v>-25.8</v>
+        <v>-24.8</v>
       </c>
       <c r="H7" t="n">
-        <v>74.09999999999999</v>
+        <v>76.3</v>
       </c>
       <c r="I7" t="n">
         <v>1904</v>
       </c>
       <c r="J7" t="n">
-        <v>0</v>
+        <v>1.3</v>
       </c>
       <c r="K7" t="n">
-        <v>1175</v>
+        <v>1330</v>
       </c>
       <c r="L7" t="n">
-        <v>-38.3</v>
+        <v>-31</v>
       </c>
       <c r="M7" t="n">
-        <v>897.5</v>
+        <v>1029</v>
       </c>
       <c r="N7" t="n">
         <v>1175</v>
       </c>
       <c r="O7" t="n">
-        <v>0</v>
+        <v>13.2</v>
       </c>
       <c r="P7" t="n">
-        <v>6496</v>
+        <v>6952</v>
       </c>
       <c r="Q7" t="n">
-        <v>117.6</v>
+        <v>132.9</v>
       </c>
       <c r="R7" t="n">
         <v>6496</v>
       </c>
       <c r="S7" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="T7" t="n">
-        <v>6105</v>
+        <v>5610</v>
       </c>
       <c r="U7" t="n">
-        <v>-6</v>
+        <v>-19.3</v>
       </c>
       <c r="V7" t="n">
         <v>6105</v>
       </c>
       <c r="W7" t="n">
-        <v>0</v>
+        <v>-8.1</v>
       </c>
       <c r="X7" t="n">
-        <v>6170</v>
+        <v>5480</v>
       </c>
       <c r="Y7" t="n">
-        <v>1.1</v>
+        <v>-2.3</v>
       </c>
       <c r="Z7" t="n">
         <v>6170</v>
       </c>
       <c r="AA7" t="n">
-        <v>0</v>
+        <v>-11.2</v>
       </c>
       <c r="AB7" t="n">
         <v>42150</v>
@@ -1670,70 +1670,70 @@
         </is>
       </c>
       <c r="F13" t="n">
-        <v>7627.1</v>
+        <v>7242.4</v>
       </c>
       <c r="G13" t="n">
-        <v>-13.9</v>
+        <v>-18.2</v>
       </c>
       <c r="H13" t="n">
-        <v>14.9</v>
+        <v>9.1</v>
       </c>
       <c r="I13" t="n">
         <v>7769.4</v>
       </c>
       <c r="J13" t="n">
-        <v>-1.8</v>
+        <v>-6.8</v>
       </c>
       <c r="K13" t="n">
-        <v>7450.9</v>
+        <v>7867</v>
       </c>
       <c r="L13" t="n">
-        <v>-2.3</v>
+        <v>8.6</v>
       </c>
       <c r="M13" t="n">
-        <v>90.40000000000001</v>
+        <v>101.1</v>
       </c>
       <c r="N13" t="n">
         <v>7188.2</v>
       </c>
       <c r="O13" t="n">
-        <v>3.7</v>
+        <v>9.4</v>
       </c>
       <c r="P13" t="n">
-        <v>32887.4</v>
+        <v>32937.6</v>
       </c>
       <c r="Q13" t="n">
-        <v>23.7</v>
+        <v>23.9</v>
       </c>
       <c r="R13" t="n">
         <v>32996.1</v>
       </c>
       <c r="S13" t="n">
-        <v>-0.3</v>
+        <v>-0.2</v>
       </c>
       <c r="T13" t="n">
-        <v>40481.2</v>
+        <v>39448.2</v>
       </c>
       <c r="U13" t="n">
-        <v>23.1</v>
+        <v>19.8</v>
       </c>
       <c r="V13" t="n">
         <v>39889.6</v>
       </c>
       <c r="W13" t="n">
-        <v>1.5</v>
+        <v>-1.1</v>
       </c>
       <c r="X13" t="n">
-        <v>39144</v>
+        <v>38291.6</v>
       </c>
       <c r="Y13" t="n">
-        <v>-3.3</v>
+        <v>-2.9</v>
       </c>
       <c r="Z13" t="n">
         <v>38638.7</v>
       </c>
       <c r="AA13" t="n">
-        <v>1.3</v>
+        <v>-0.9</v>
       </c>
       <c r="AB13" t="n">
         <v>602000</v>
@@ -3135,25 +3135,25 @@
         </is>
       </c>
       <c r="F28" t="n">
-        <v>1852.8</v>
+        <v>1846.6</v>
       </c>
       <c r="G28" t="n">
-        <v>5.2</v>
+        <v>4.8</v>
       </c>
       <c r="H28" t="n">
-        <v>41.5</v>
+        <v>41.1</v>
       </c>
       <c r="I28" t="n">
         <v>1868.1</v>
       </c>
       <c r="J28" t="n">
-        <v>-0.8</v>
+        <v>-1.2</v>
       </c>
       <c r="K28" t="n">
         <v>1889.8</v>
       </c>
       <c r="L28" t="n">
-        <v>2</v>
+        <v>2.3</v>
       </c>
       <c r="M28" t="n">
         <v>35.8</v>
@@ -3165,40 +3165,40 @@
         <v>-0.1</v>
       </c>
       <c r="P28" t="n">
-        <v>7275.4</v>
+        <v>7269.2</v>
       </c>
       <c r="Q28" t="n">
-        <v>38.8</v>
+        <v>38.7</v>
       </c>
       <c r="R28" t="n">
         <v>7293.4</v>
       </c>
       <c r="S28" t="n">
-        <v>-0.2</v>
+        <v>-0.3</v>
       </c>
       <c r="T28" t="n">
-        <v>8922.6</v>
+        <v>8941.799999999999</v>
       </c>
       <c r="U28" t="n">
-        <v>22.6</v>
+        <v>23</v>
       </c>
       <c r="V28" t="n">
         <v>8941.799999999999</v>
       </c>
       <c r="W28" t="n">
-        <v>-0.2</v>
+        <v>0</v>
       </c>
       <c r="X28" t="n">
-        <v>10608.5</v>
+        <v>10639.5</v>
       </c>
       <c r="Y28" t="n">
-        <v>18.9</v>
+        <v>19</v>
       </c>
       <c r="Z28" t="n">
         <v>10594.4</v>
       </c>
       <c r="AA28" t="n">
-        <v>0.1</v>
+        <v>0.4</v>
       </c>
       <c r="AB28" t="n">
         <v>1225000</v>
@@ -3855,64 +3855,64 @@
         </is>
       </c>
       <c r="F35" t="n">
-        <v>614.2</v>
+        <v>611.7</v>
       </c>
       <c r="G35" t="n">
-        <v>3.7</v>
+        <v>3.2</v>
       </c>
       <c r="H35" t="n">
-        <v>12.9</v>
+        <v>12.5</v>
       </c>
       <c r="I35" t="n">
         <v>622.4</v>
       </c>
       <c r="J35" t="n">
-        <v>-1.3</v>
+        <v>-1.7</v>
       </c>
       <c r="K35" t="n">
-        <v>439.8</v>
+        <v>435.7</v>
       </c>
       <c r="L35" t="n">
-        <v>-28.4</v>
+        <v>-28.8</v>
       </c>
       <c r="M35" t="n">
-        <v>31.9</v>
+        <v>30.6</v>
       </c>
       <c r="N35" t="n">
         <v>439.9</v>
       </c>
       <c r="O35" t="n">
-        <v>-0</v>
+        <v>-1</v>
       </c>
       <c r="P35" t="n">
-        <v>2321.2</v>
+        <v>2314.5</v>
       </c>
       <c r="Q35" t="n">
-        <v>26.2</v>
+        <v>25.8</v>
       </c>
       <c r="R35" t="n">
         <v>2329.5</v>
       </c>
       <c r="S35" t="n">
-        <v>-0.4</v>
+        <v>-0.6</v>
       </c>
       <c r="T35" t="n">
-        <v>2477.2</v>
+        <v>2474.2</v>
       </c>
       <c r="U35" t="n">
-        <v>6.7</v>
+        <v>6.9</v>
       </c>
       <c r="V35" t="n">
         <v>2484</v>
       </c>
       <c r="W35" t="n">
-        <v>-0.3</v>
+        <v>-0.4</v>
       </c>
       <c r="X35" t="n">
         <v>2636.4</v>
       </c>
       <c r="Y35" t="n">
-        <v>6.4</v>
+        <v>6.6</v>
       </c>
       <c r="Z35" t="n">
         <v>2648</v>
@@ -4063,25 +4063,25 @@
         </is>
       </c>
       <c r="F37" t="n">
-        <v>834.5</v>
+        <v>828</v>
       </c>
       <c r="G37" t="n">
-        <v>49.4</v>
+        <v>48.3</v>
       </c>
       <c r="H37" t="n">
-        <v>-9.1</v>
+        <v>-9.800000000000001</v>
       </c>
       <c r="I37" t="n">
         <v>841.2</v>
       </c>
       <c r="J37" t="n">
-        <v>-0.8</v>
+        <v>-1.6</v>
       </c>
       <c r="K37" t="n">
-        <v>91.59999999999999</v>
+        <v>90.2</v>
       </c>
       <c r="L37" t="n">
-        <v>-89</v>
+        <v>-89.09999999999999</v>
       </c>
       <c r="M37" t="inlineStr">
         <is>
@@ -4092,37 +4092,37 @@
         <v>92.8</v>
       </c>
       <c r="O37" t="n">
-        <v>-1.3</v>
+        <v>-2.8</v>
       </c>
       <c r="P37" t="n">
-        <v>1968.9</v>
+        <v>1961</v>
       </c>
       <c r="Q37" t="n">
-        <v>17.8</v>
+        <v>17.3</v>
       </c>
       <c r="R37" t="n">
         <v>1976.6</v>
       </c>
       <c r="S37" t="n">
-        <v>-0.4</v>
+        <v>-0.8</v>
       </c>
       <c r="T37" t="n">
-        <v>2212.4</v>
+        <v>2203</v>
       </c>
       <c r="U37" t="n">
-        <v>12.4</v>
+        <v>12.3</v>
       </c>
       <c r="V37" t="n">
         <v>2222.8</v>
       </c>
       <c r="W37" t="n">
-        <v>-0.5</v>
+        <v>-0.9</v>
       </c>
       <c r="X37" t="n">
         <v>2381.8</v>
       </c>
       <c r="Y37" t="n">
-        <v>7.7</v>
+        <v>8.1</v>
       </c>
       <c r="Z37" t="n">
         <v>2388.1</v>
@@ -4221,16 +4221,16 @@
         <v>-0.7</v>
       </c>
       <c r="X38" t="n">
-        <v>125630.7</v>
+        <v>125691.5</v>
       </c>
       <c r="Y38" t="n">
-        <v>8.300000000000001</v>
+        <v>8.4</v>
       </c>
       <c r="Z38" t="n">
         <v>127535</v>
       </c>
       <c r="AA38" t="n">
-        <v>-1.5</v>
+        <v>-1.4</v>
       </c>
       <c r="AB38" t="n">
         <v>293000</v>
@@ -4677,25 +4677,25 @@
         </is>
       </c>
       <c r="F43" t="n">
-        <v>5109.6</v>
+        <v>5092.6</v>
       </c>
       <c r="G43" t="n">
-        <v>-25</v>
+        <v>-25.2</v>
       </c>
       <c r="H43" t="n">
-        <v>30.6</v>
+        <v>30.1</v>
       </c>
       <c r="I43" t="n">
         <v>5184.6</v>
       </c>
       <c r="J43" t="n">
-        <v>-1.4</v>
+        <v>-1.8</v>
       </c>
       <c r="K43" t="n">
         <v>4370.3</v>
       </c>
       <c r="L43" t="n">
-        <v>-14.5</v>
+        <v>-14.2</v>
       </c>
       <c r="M43" t="n">
         <v>4.5</v>
@@ -6173,13 +6173,13 @@
         </is>
       </c>
       <c r="F58" t="n">
-        <v>6453.9</v>
+        <v>6453.3</v>
       </c>
       <c r="G58" t="n">
-        <v>46.6</v>
+        <v>46.5</v>
       </c>
       <c r="H58" t="n">
-        <v>148</v>
+        <v>147.9</v>
       </c>
       <c r="I58" t="n">
         <v>6422.7</v>
@@ -6188,55 +6188,55 @@
         <v>0.5</v>
       </c>
       <c r="K58" t="n">
-        <v>6974.6</v>
+        <v>7023.4</v>
       </c>
       <c r="L58" t="n">
-        <v>8.1</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="M58" t="n">
-        <v>191.2</v>
+        <v>193.3</v>
       </c>
       <c r="N58" t="n">
         <v>6829.6</v>
       </c>
       <c r="O58" t="n">
-        <v>2.1</v>
+        <v>2.8</v>
       </c>
       <c r="P58" t="n">
-        <v>20637.5</v>
+        <v>20685.6</v>
       </c>
       <c r="Q58" t="n">
-        <v>126</v>
+        <v>126.5</v>
       </c>
       <c r="R58" t="n">
         <v>20461.4</v>
       </c>
       <c r="S58" t="n">
-        <v>0.9</v>
+        <v>1.1</v>
       </c>
       <c r="T58" t="n">
-        <v>41087.1</v>
+        <v>41627.4</v>
       </c>
       <c r="U58" t="n">
-        <v>99.09999999999999</v>
+        <v>101.2</v>
       </c>
       <c r="V58" t="n">
         <v>40214.8</v>
       </c>
       <c r="W58" t="n">
-        <v>2.2</v>
+        <v>3.5</v>
       </c>
       <c r="X58" t="n">
-        <v>64033.9</v>
+        <v>64992.1</v>
       </c>
       <c r="Y58" t="n">
-        <v>55.8</v>
+        <v>56.1</v>
       </c>
       <c r="Z58" t="n">
         <v>62301</v>
       </c>
       <c r="AA58" t="n">
-        <v>2.8</v>
+        <v>4.3</v>
       </c>
       <c r="AB58" t="n">
         <v>1111000</v>
@@ -6708,55 +6708,55 @@
         <v>0</v>
       </c>
       <c r="K63" t="n">
-        <v>2410.4</v>
+        <v>2414.5</v>
       </c>
       <c r="L63" t="n">
-        <v>24.3</v>
+        <v>24.5</v>
       </c>
       <c r="M63" t="n">
-        <v>85.8</v>
+        <v>86.09999999999999</v>
       </c>
       <c r="N63" t="n">
         <v>2208.8</v>
       </c>
       <c r="O63" t="n">
-        <v>9.1</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="P63" t="n">
-        <v>7668.6</v>
+        <v>7693.8</v>
       </c>
       <c r="Q63" t="n">
-        <v>79.8</v>
+        <v>80.40000000000001</v>
       </c>
       <c r="R63" t="n">
         <v>7217</v>
       </c>
       <c r="S63" t="n">
-        <v>6.3</v>
+        <v>6.6</v>
       </c>
       <c r="T63" t="n">
-        <v>11238.2</v>
+        <v>11248.2</v>
       </c>
       <c r="U63" t="n">
-        <v>46.5</v>
+        <v>46.2</v>
       </c>
       <c r="V63" t="n">
         <v>10444.5</v>
       </c>
       <c r="W63" t="n">
-        <v>7.6</v>
+        <v>7.7</v>
       </c>
       <c r="X63" t="n">
-        <v>14699.9</v>
+        <v>14718.4</v>
       </c>
       <c r="Y63" t="n">
-        <v>30.8</v>
+        <v>30.9</v>
       </c>
       <c r="Z63" t="n">
         <v>13854.9</v>
       </c>
       <c r="AA63" t="n">
-        <v>6.1</v>
+        <v>6.2</v>
       </c>
       <c r="AB63" t="n">
         <v>154600</v>
@@ -7258,70 +7258,70 @@
         </is>
       </c>
       <c r="F69" t="n">
-        <v>2028.9</v>
+        <v>1972.8</v>
       </c>
       <c r="G69" t="n">
-        <v>-17.4</v>
+        <v>-19.7</v>
       </c>
       <c r="H69" t="n">
-        <v>-0.4</v>
+        <v>-3.2</v>
       </c>
       <c r="I69" t="n">
         <v>2028.9</v>
       </c>
       <c r="J69" t="n">
-        <v>0</v>
+        <v>-2.8</v>
       </c>
       <c r="K69" t="n">
-        <v>3867.2</v>
+        <v>3825.4</v>
       </c>
       <c r="L69" t="n">
-        <v>90.59999999999999</v>
+        <v>93.90000000000001</v>
       </c>
       <c r="M69" t="n">
-        <v>19.1</v>
+        <v>17.8</v>
       </c>
       <c r="N69" t="n">
         <v>3867.2</v>
       </c>
       <c r="O69" t="n">
-        <v>0</v>
+        <v>-1.1</v>
       </c>
       <c r="P69" t="n">
-        <v>11250.8</v>
+        <v>11155.8</v>
       </c>
       <c r="Q69" t="n">
-        <v>69.2</v>
+        <v>67.8</v>
       </c>
       <c r="R69" t="n">
         <v>11250.8</v>
       </c>
       <c r="S69" t="n">
-        <v>0</v>
+        <v>-0.8</v>
       </c>
       <c r="T69" t="n">
-        <v>13798.7</v>
+        <v>13706.8</v>
       </c>
       <c r="U69" t="n">
-        <v>22.6</v>
+        <v>22.9</v>
       </c>
       <c r="V69" t="n">
         <v>13798.7</v>
       </c>
       <c r="W69" t="n">
-        <v>0</v>
+        <v>-0.7</v>
       </c>
       <c r="X69" t="n">
-        <v>16417.9</v>
+        <v>16345.5</v>
       </c>
       <c r="Y69" t="n">
-        <v>19</v>
+        <v>19.3</v>
       </c>
       <c r="Z69" t="n">
         <v>16417.9</v>
       </c>
       <c r="AA69" t="n">
-        <v>0</v>
+        <v>-0.4</v>
       </c>
       <c r="AB69" t="n">
         <v>376000</v>
@@ -7474,70 +7474,70 @@
         </is>
       </c>
       <c r="F71" t="n">
-        <v>7792.3</v>
+        <v>7975.3</v>
       </c>
       <c r="G71" t="n">
-        <v>120</v>
+        <v>125.2</v>
       </c>
       <c r="H71" t="n">
-        <v>162.5</v>
+        <v>168.7</v>
       </c>
       <c r="I71" t="n">
         <v>7442.9</v>
       </c>
       <c r="J71" t="n">
-        <v>4.7</v>
+        <v>7.2</v>
       </c>
       <c r="K71" t="n">
-        <v>5997.8</v>
+        <v>6091.3</v>
       </c>
       <c r="L71" t="n">
-        <v>-23</v>
+        <v>-23.6</v>
       </c>
       <c r="M71" t="n">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="N71" t="n">
         <v>5493.4</v>
       </c>
       <c r="O71" t="n">
-        <v>9.199999999999999</v>
+        <v>10.9</v>
       </c>
       <c r="P71" t="n">
-        <v>20059.7</v>
+        <v>20301.2</v>
       </c>
       <c r="Q71" t="n">
-        <v>37.3</v>
+        <v>38.9</v>
       </c>
       <c r="R71" t="n">
         <v>19208.9</v>
       </c>
       <c r="S71" t="n">
-        <v>4.4</v>
+        <v>5.7</v>
       </c>
       <c r="T71" t="n">
-        <v>13318.2</v>
+        <v>13306.5</v>
       </c>
       <c r="U71" t="n">
-        <v>-33.6</v>
+        <v>-34.5</v>
       </c>
       <c r="V71" t="n">
         <v>12894.5</v>
       </c>
       <c r="W71" t="n">
-        <v>3.3</v>
+        <v>3.2</v>
       </c>
       <c r="X71" t="n">
-        <v>9981.9</v>
+        <v>9830.9</v>
       </c>
       <c r="Y71" t="n">
-        <v>-25.1</v>
+        <v>-26.1</v>
       </c>
       <c r="Z71" t="n">
         <v>9921</v>
       </c>
       <c r="AA71" t="n">
-        <v>0.6</v>
+        <v>-0.9</v>
       </c>
       <c r="AB71" t="n">
         <v>22500</v>
@@ -8507,34 +8507,34 @@
         </is>
       </c>
       <c r="F81" t="n">
-        <v>142</v>
+        <v>124</v>
       </c>
       <c r="G81" t="n">
-        <v>41.9</v>
+        <v>23.9</v>
       </c>
       <c r="H81" t="n">
-        <v>21.1</v>
+        <v>5.7</v>
       </c>
       <c r="I81" t="n">
         <v>142</v>
       </c>
       <c r="J81" t="n">
-        <v>0</v>
+        <v>-12.7</v>
       </c>
       <c r="K81" t="n">
-        <v>163</v>
+        <v>146</v>
       </c>
       <c r="L81" t="n">
-        <v>14.8</v>
+        <v>17.7</v>
       </c>
       <c r="M81" t="n">
-        <v>87.09999999999999</v>
+        <v>67.59999999999999</v>
       </c>
       <c r="N81" t="n">
         <v>163</v>
       </c>
       <c r="O81" t="n">
-        <v>0</v>
+        <v>-10.4</v>
       </c>
       <c r="P81" t="n">
         <v>488</v>
@@ -8609,70 +8609,70 @@
         </is>
       </c>
       <c r="F82" t="n">
-        <v>513.5</v>
+        <v>507</v>
       </c>
       <c r="G82" t="n">
-        <v>3.2</v>
+        <v>1.9</v>
       </c>
       <c r="H82" t="n">
-        <v>5.2</v>
+        <v>3.9</v>
       </c>
       <c r="I82" t="n">
         <v>513.5</v>
       </c>
       <c r="J82" t="n">
-        <v>0</v>
+        <v>-1.3</v>
       </c>
       <c r="K82" t="n">
-        <v>331</v>
+        <v>329.5</v>
       </c>
       <c r="L82" t="n">
-        <v>-35.5</v>
+        <v>-35</v>
       </c>
       <c r="M82" t="n">
-        <v>96.09999999999999</v>
+        <v>95.2</v>
       </c>
       <c r="N82" t="n">
         <v>331</v>
       </c>
       <c r="O82" t="n">
-        <v>0</v>
+        <v>-0.5</v>
       </c>
       <c r="P82" t="n">
-        <v>1789.3</v>
+        <v>1781.5</v>
       </c>
       <c r="Q82" t="n">
-        <v>14.5</v>
+        <v>14</v>
       </c>
       <c r="R82" t="n">
         <v>1789.3</v>
       </c>
       <c r="S82" t="n">
-        <v>0</v>
+        <v>-0.4</v>
       </c>
       <c r="T82" t="n">
-        <v>2256.7</v>
+        <v>2248.2</v>
       </c>
       <c r="U82" t="n">
-        <v>26.1</v>
+        <v>26.2</v>
       </c>
       <c r="V82" t="n">
         <v>2256.7</v>
       </c>
       <c r="W82" t="n">
-        <v>0</v>
+        <v>-0.4</v>
       </c>
       <c r="X82" t="n">
-        <v>2968.2</v>
+        <v>2848.5</v>
       </c>
       <c r="Y82" t="n">
-        <v>31.5</v>
+        <v>26.7</v>
       </c>
       <c r="Z82" t="n">
         <v>2968.2</v>
       </c>
       <c r="AA82" t="n">
-        <v>0</v>
+        <v>-4</v>
       </c>
       <c r="AB82" t="n">
         <v>210500</v>
@@ -9047,19 +9047,19 @@
         <v>0</v>
       </c>
       <c r="P86" t="n">
-        <v>19580.1</v>
+        <v>19568.9</v>
       </c>
       <c r="Q86" t="n">
-        <v>82.40000000000001</v>
+        <v>82.3</v>
       </c>
       <c r="R86" t="n">
         <v>19580.1</v>
       </c>
       <c r="S86" t="n">
-        <v>0</v>
+        <v>-0.1</v>
       </c>
       <c r="T86" t="n">
-        <v>20854.6</v>
+        <v>20845.9</v>
       </c>
       <c r="U86" t="n">
         <v>6.5</v>
@@ -9068,19 +9068,19 @@
         <v>20854.6</v>
       </c>
       <c r="W86" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="X86" t="n">
-        <v>22206.7</v>
+        <v>22188.2</v>
       </c>
       <c r="Y86" t="n">
-        <v>6.5</v>
+        <v>6.4</v>
       </c>
       <c r="Z86" t="n">
         <v>22206.7</v>
       </c>
       <c r="AA86" t="n">
-        <v>0</v>
+        <v>-0.1</v>
       </c>
       <c r="AB86" t="n">
         <v>74200</v>
@@ -9323,70 +9323,70 @@
         </is>
       </c>
       <c r="F89" t="n">
-        <v>1113.4</v>
+        <v>1107.7</v>
       </c>
       <c r="G89" t="n">
-        <v>7.4</v>
+        <v>6.8</v>
       </c>
       <c r="H89" t="n">
-        <v>16.8</v>
+        <v>16.2</v>
       </c>
       <c r="I89" t="n">
         <v>1108.9</v>
       </c>
       <c r="J89" t="n">
-        <v>0.4</v>
+        <v>-0.1</v>
       </c>
       <c r="K89" t="n">
-        <v>1185.7</v>
+        <v>1192.3</v>
       </c>
       <c r="L89" t="n">
-        <v>6.5</v>
+        <v>7.6</v>
       </c>
       <c r="M89" t="n">
-        <v>32.2</v>
+        <v>32.9</v>
       </c>
       <c r="N89" t="n">
         <v>1184.7</v>
       </c>
       <c r="O89" t="n">
-        <v>0.1</v>
+        <v>0.6</v>
       </c>
       <c r="P89" t="n">
-        <v>4324</v>
+        <v>4307.8</v>
       </c>
       <c r="Q89" t="n">
-        <v>59.9</v>
+        <v>59.3</v>
       </c>
       <c r="R89" t="n">
         <v>4318.2</v>
       </c>
       <c r="S89" t="n">
-        <v>0.1</v>
+        <v>-0.2</v>
       </c>
       <c r="T89" t="n">
-        <v>4984.4</v>
+        <v>4936.2</v>
       </c>
       <c r="U89" t="n">
-        <v>15.3</v>
+        <v>14.6</v>
       </c>
       <c r="V89" t="n">
         <v>4982.1</v>
       </c>
       <c r="W89" t="n">
-        <v>0</v>
+        <v>-0.9</v>
       </c>
       <c r="X89" t="n">
-        <v>5543.8</v>
+        <v>5509.4</v>
       </c>
       <c r="Y89" t="n">
-        <v>11.2</v>
+        <v>11.6</v>
       </c>
       <c r="Z89" t="n">
         <v>5541.6</v>
       </c>
       <c r="AA89" t="n">
-        <v>0</v>
+        <v>-0.6</v>
       </c>
       <c r="AB89" t="n">
         <v>3690</v>
@@ -9578,34 +9578,34 @@
         </is>
       </c>
       <c r="F92" t="n">
-        <v>84</v>
+        <v>118</v>
       </c>
       <c r="G92" t="n">
-        <v>16.5</v>
+        <v>63.7</v>
       </c>
       <c r="H92" t="n">
-        <v>-27.4</v>
+        <v>2</v>
       </c>
       <c r="I92" t="n">
         <v>84</v>
       </c>
       <c r="J92" t="n">
-        <v>0</v>
+        <v>40.5</v>
       </c>
       <c r="K92" t="n">
-        <v>165.5</v>
+        <v>141</v>
       </c>
       <c r="L92" t="n">
-        <v>97</v>
+        <v>19.5</v>
       </c>
       <c r="M92" t="n">
-        <v>36.7</v>
+        <v>16.4</v>
       </c>
       <c r="N92" t="n">
         <v>165.5</v>
       </c>
       <c r="O92" t="n">
-        <v>0</v>
+        <v>-14.8</v>
       </c>
       <c r="P92" t="n">
         <v>452.5</v>
@@ -9899,55 +9899,55 @@
         <v>0</v>
       </c>
       <c r="K95" t="n">
-        <v>2786</v>
+        <v>4172.8</v>
       </c>
       <c r="L95" t="n">
-        <v>11.8</v>
+        <v>67.40000000000001</v>
       </c>
       <c r="M95" t="n">
-        <v>0.4</v>
+        <v>50.4</v>
       </c>
       <c r="N95" t="n">
         <v>2763.3</v>
       </c>
       <c r="O95" t="n">
-        <v>0.8</v>
+        <v>51</v>
       </c>
       <c r="P95" t="n">
-        <v>9893.1</v>
+        <v>13535.9</v>
       </c>
       <c r="Q95" t="n">
-        <v>24.9</v>
+        <v>70.90000000000001</v>
       </c>
       <c r="R95" t="n">
         <v>9818.9</v>
       </c>
       <c r="S95" t="n">
-        <v>0.8</v>
+        <v>37.9</v>
       </c>
       <c r="T95" t="n">
-        <v>12058.4</v>
+        <v>14373.8</v>
       </c>
       <c r="U95" t="n">
-        <v>21.9</v>
+        <v>6.2</v>
       </c>
       <c r="V95" t="n">
         <v>11945.8</v>
       </c>
       <c r="W95" t="n">
-        <v>0.9</v>
+        <v>20.3</v>
       </c>
       <c r="X95" t="n">
-        <v>13525.4</v>
+        <v>15696.5</v>
       </c>
       <c r="Y95" t="n">
-        <v>12.2</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="Z95" t="n">
         <v>13290.1</v>
       </c>
       <c r="AA95" t="n">
-        <v>1.8</v>
+        <v>18.1</v>
       </c>
       <c r="AB95" t="n">
         <v>59100</v>
@@ -9986,37 +9986,37 @@
         </is>
       </c>
       <c r="F96" t="n">
-        <v>9945.799999999999</v>
+        <v>10033.4</v>
       </c>
       <c r="G96" t="n">
-        <v>-3.6</v>
+        <v>-2.8</v>
       </c>
       <c r="H96" t="n">
-        <v>0.1</v>
+        <v>1</v>
       </c>
       <c r="I96" t="n">
         <v>9943.1</v>
       </c>
       <c r="J96" t="n">
-        <v>0</v>
+        <v>0.9</v>
       </c>
       <c r="K96" t="n">
-        <v>10556.6</v>
+        <v>10375.6</v>
       </c>
       <c r="L96" t="n">
-        <v>6.1</v>
+        <v>3.4</v>
       </c>
       <c r="M96" t="n">
-        <v>28.4</v>
+        <v>26.2</v>
       </c>
       <c r="N96" t="n">
         <v>10529.9</v>
       </c>
       <c r="O96" t="n">
-        <v>0.3</v>
+        <v>-1.5</v>
       </c>
       <c r="P96" t="n">
-        <v>37919.8</v>
+        <v>37936.5</v>
       </c>
       <c r="Q96" t="n">
         <v>15.2</v>
@@ -10028,28 +10028,28 @@
         <v>0.1</v>
       </c>
       <c r="T96" t="n">
-        <v>43987.6</v>
+        <v>44061.4</v>
       </c>
       <c r="U96" t="n">
-        <v>16</v>
+        <v>16.1</v>
       </c>
       <c r="V96" t="n">
         <v>44032.6</v>
       </c>
       <c r="W96" t="n">
-        <v>-0.1</v>
+        <v>0.1</v>
       </c>
       <c r="X96" t="n">
-        <v>47719.1</v>
+        <v>47656.2</v>
       </c>
       <c r="Y96" t="n">
-        <v>8.5</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="Z96" t="n">
         <v>47685.8</v>
       </c>
       <c r="AA96" t="n">
-        <v>0.1</v>
+        <v>-0.1</v>
       </c>
       <c r="AB96" t="n">
         <v>286000</v>
@@ -10088,13 +10088,13 @@
         </is>
       </c>
       <c r="F97" t="n">
-        <v>1900.4</v>
+        <v>1899.6</v>
       </c>
       <c r="G97" t="n">
         <v>-1.9</v>
       </c>
       <c r="H97" t="n">
-        <v>51.8</v>
+        <v>51.7</v>
       </c>
       <c r="I97" t="n">
         <v>1879.6</v>
@@ -10103,22 +10103,22 @@
         <v>1.1</v>
       </c>
       <c r="K97" t="n">
-        <v>1753.8</v>
+        <v>1755.2</v>
       </c>
       <c r="L97" t="n">
-        <v>-7.7</v>
+        <v>-7.6</v>
       </c>
       <c r="M97" t="n">
-        <v>34.5</v>
+        <v>34.6</v>
       </c>
       <c r="N97" t="n">
         <v>1721.6</v>
       </c>
       <c r="O97" t="n">
-        <v>1.9</v>
+        <v>2</v>
       </c>
       <c r="P97" t="n">
-        <v>6999.5</v>
+        <v>7000.2</v>
       </c>
       <c r="Q97" t="n">
         <v>42.3</v>
@@ -10130,28 +10130,28 @@
         <v>0.8</v>
       </c>
       <c r="T97" t="n">
-        <v>7302</v>
+        <v>7320.6</v>
       </c>
       <c r="U97" t="n">
-        <v>4.3</v>
+        <v>4.6</v>
       </c>
       <c r="V97" t="n">
         <v>7183.4</v>
       </c>
       <c r="W97" t="n">
-        <v>1.7</v>
+        <v>1.9</v>
       </c>
       <c r="X97" t="n">
-        <v>7379.1</v>
+        <v>7419.9</v>
       </c>
       <c r="Y97" t="n">
-        <v>1.1</v>
+        <v>1.4</v>
       </c>
       <c r="Z97" t="n">
         <v>7259.9</v>
       </c>
       <c r="AA97" t="n">
-        <v>1.6</v>
+        <v>2.2</v>
       </c>
       <c r="AB97" t="n">
         <v>6190</v>
@@ -10598,19 +10598,19 @@
         </is>
       </c>
       <c r="F102" t="n">
-        <v>461</v>
+        <v>446</v>
       </c>
       <c r="G102" t="n">
-        <v>-11.2</v>
+        <v>-14.1</v>
       </c>
       <c r="H102" t="n">
-        <v>-13</v>
+        <v>-15.8</v>
       </c>
       <c r="I102" t="n">
         <v>494</v>
       </c>
       <c r="J102" t="n">
-        <v>-6.7</v>
+        <v>-9.699999999999999</v>
       </c>
       <c r="AB102" t="n">
         <v>10660</v>
@@ -10691,19 +10691,19 @@
         <v>-0.1</v>
       </c>
       <c r="T103" t="n">
-        <v>12248</v>
+        <v>12236.9</v>
       </c>
       <c r="U103" t="n">
-        <v>6.6</v>
+        <v>6.5</v>
       </c>
       <c r="V103" t="n">
         <v>12320.2</v>
       </c>
       <c r="W103" t="n">
-        <v>-0.6</v>
+        <v>-0.7</v>
       </c>
       <c r="X103" t="n">
-        <v>13178.1</v>
+        <v>13167</v>
       </c>
       <c r="Y103" t="n">
         <v>7.6</v>
@@ -10712,7 +10712,7 @@
         <v>13250.9</v>
       </c>
       <c r="AA103" t="n">
-        <v>-0.5</v>
+        <v>-0.6</v>
       </c>
       <c r="AB103" t="n">
         <v>14200</v>
@@ -10955,25 +10955,25 @@
         </is>
       </c>
       <c r="F106" t="n">
-        <v>5063.1</v>
+        <v>5077.8</v>
       </c>
       <c r="G106" t="n">
-        <v>22.2</v>
+        <v>22.5</v>
       </c>
       <c r="H106" t="n">
-        <v>8.800000000000001</v>
+        <v>9.1</v>
       </c>
       <c r="I106" t="n">
         <v>4994.6</v>
       </c>
       <c r="J106" t="n">
-        <v>1.4</v>
+        <v>1.7</v>
       </c>
       <c r="K106" t="n">
-        <v>2487.9</v>
+        <v>2486.7</v>
       </c>
       <c r="L106" t="n">
-        <v>-50.9</v>
+        <v>-51</v>
       </c>
       <c r="M106" t="n">
         <v>2.4</v>
@@ -10985,22 +10985,22 @@
         <v>-2.2</v>
       </c>
       <c r="P106" t="n">
-        <v>15340.1</v>
+        <v>15353.6</v>
       </c>
       <c r="Q106" t="n">
-        <v>14.2</v>
+        <v>14.3</v>
       </c>
       <c r="R106" t="n">
         <v>15327.6</v>
       </c>
       <c r="S106" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="T106" t="n">
-        <v>16490.3</v>
+        <v>16485.1</v>
       </c>
       <c r="U106" t="n">
-        <v>7.5</v>
+        <v>7.4</v>
       </c>
       <c r="V106" t="n">
         <v>16550</v>
@@ -11012,7 +11012,7 @@
         <v>17402.8</v>
       </c>
       <c r="Y106" t="n">
-        <v>5.5</v>
+        <v>5.6</v>
       </c>
       <c r="Z106" t="n">
         <v>17515.4</v>
@@ -11176,55 +11176,55 @@
         <v>0</v>
       </c>
       <c r="K108" t="n">
-        <v>3110.1</v>
+        <v>2967.7</v>
       </c>
       <c r="L108" t="n">
-        <v>15</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="M108" t="n">
-        <v>84.59999999999999</v>
+        <v>76.09999999999999</v>
       </c>
       <c r="N108" t="n">
         <v>3181.6</v>
       </c>
       <c r="O108" t="n">
-        <v>-2.2</v>
+        <v>-6.7</v>
       </c>
       <c r="P108" t="n">
-        <v>6093.7</v>
+        <v>5808.8</v>
       </c>
       <c r="Q108" t="n">
-        <v>17.9</v>
+        <v>12.4</v>
       </c>
       <c r="R108" t="n">
         <v>6280.9</v>
       </c>
       <c r="S108" t="n">
-        <v>-3</v>
+        <v>-7.5</v>
       </c>
       <c r="T108" t="n">
-        <v>9957.4</v>
+        <v>9510</v>
       </c>
       <c r="U108" t="n">
-        <v>63.4</v>
+        <v>63.7</v>
       </c>
       <c r="V108" t="n">
         <v>10410.3</v>
       </c>
       <c r="W108" t="n">
-        <v>-4.4</v>
+        <v>-8.6</v>
       </c>
       <c r="X108" t="n">
-        <v>12623.9</v>
+        <v>12667.3</v>
       </c>
       <c r="Y108" t="n">
-        <v>26.8</v>
+        <v>33.2</v>
       </c>
       <c r="Z108" t="n">
         <v>13102.4</v>
       </c>
       <c r="AA108" t="n">
-        <v>-3.7</v>
+        <v>-3.3</v>
       </c>
       <c r="AB108" t="n">
         <v>7100</v>
@@ -11263,70 +11263,70 @@
         </is>
       </c>
       <c r="F109" t="n">
-        <v>531.8</v>
+        <v>540.4</v>
       </c>
       <c r="G109" t="n">
-        <v>49.6</v>
+        <v>52</v>
       </c>
       <c r="H109" t="n">
-        <v>34.6</v>
+        <v>36.8</v>
       </c>
       <c r="I109" t="n">
         <v>523.4</v>
       </c>
       <c r="J109" t="n">
-        <v>1.6</v>
+        <v>3.2</v>
       </c>
       <c r="K109" t="n">
-        <v>330.2</v>
+        <v>320.2</v>
       </c>
       <c r="L109" t="n">
-        <v>-37.9</v>
+        <v>-40.7</v>
       </c>
       <c r="M109" t="n">
-        <v>104.1</v>
+        <v>97.90000000000001</v>
       </c>
       <c r="N109" t="n">
         <v>334.6</v>
       </c>
       <c r="O109" t="n">
-        <v>-1.3</v>
+        <v>-4.3</v>
       </c>
       <c r="P109" t="n">
-        <v>1656.6</v>
+        <v>1649.6</v>
       </c>
       <c r="Q109" t="n">
-        <v>6.3</v>
+        <v>5.9</v>
       </c>
       <c r="R109" t="n">
         <v>1660.7</v>
       </c>
       <c r="S109" t="n">
-        <v>-0.2</v>
+        <v>-0.7</v>
       </c>
       <c r="T109" t="n">
-        <v>2013.4</v>
+        <v>2011.3</v>
       </c>
       <c r="U109" t="n">
-        <v>21.5</v>
+        <v>21.9</v>
       </c>
       <c r="V109" t="n">
         <v>2011.6</v>
       </c>
       <c r="W109" t="n">
-        <v>0.1</v>
+        <v>-0</v>
       </c>
       <c r="X109" t="n">
-        <v>2334</v>
+        <v>2314.7</v>
       </c>
       <c r="Y109" t="n">
-        <v>15.9</v>
+        <v>15.1</v>
       </c>
       <c r="Z109" t="n">
         <v>2334</v>
       </c>
       <c r="AA109" t="n">
-        <v>0</v>
+        <v>-0.8</v>
       </c>
       <c r="AB109" t="n">
         <v>9590</v>
@@ -11467,70 +11467,70 @@
         </is>
       </c>
       <c r="F111" t="n">
-        <v>636.4</v>
+        <v>636.9</v>
       </c>
       <c r="G111" t="n">
-        <v>45.3</v>
+        <v>45.4</v>
       </c>
       <c r="H111" t="n">
-        <v>-12.5</v>
+        <v>-12.4</v>
       </c>
       <c r="I111" t="n">
         <v>636.4</v>
       </c>
       <c r="J111" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="K111" t="n">
-        <v>313.4</v>
+        <v>309.2</v>
       </c>
       <c r="L111" t="n">
-        <v>-50.8</v>
+        <v>-51.5</v>
       </c>
       <c r="M111" t="n">
-        <v>5.1</v>
+        <v>3.7</v>
       </c>
       <c r="N111" t="n">
         <v>313.4</v>
       </c>
       <c r="O111" t="n">
-        <v>0</v>
+        <v>-1.3</v>
       </c>
       <c r="P111" t="n">
-        <v>2115.2</v>
+        <v>2108</v>
       </c>
       <c r="Q111" t="n">
-        <v>-10.1</v>
+        <v>-10.4</v>
       </c>
       <c r="R111" t="n">
         <v>2115.2</v>
       </c>
       <c r="S111" t="n">
-        <v>0</v>
+        <v>-0.3</v>
       </c>
       <c r="T111" t="n">
-        <v>2048.5</v>
+        <v>2026.4</v>
       </c>
       <c r="U111" t="n">
-        <v>-3.2</v>
+        <v>-3.9</v>
       </c>
       <c r="V111" t="n">
         <v>2048.5</v>
       </c>
       <c r="W111" t="n">
-        <v>0</v>
+        <v>-1.1</v>
       </c>
       <c r="X111" t="n">
-        <v>2640.3</v>
+        <v>2576</v>
       </c>
       <c r="Y111" t="n">
-        <v>28.9</v>
+        <v>27.1</v>
       </c>
       <c r="Z111" t="n">
         <v>2640.3</v>
       </c>
       <c r="AA111" t="n">
-        <v>0</v>
+        <v>-2.4</v>
       </c>
       <c r="AB111" t="n">
         <v>14170</v>
@@ -12714,70 +12714,70 @@
         </is>
       </c>
       <c r="F124" t="n">
-        <v>382.7</v>
+        <v>380.3</v>
       </c>
       <c r="G124" t="n">
-        <v>-27.6</v>
+        <v>-28.1</v>
       </c>
       <c r="H124" t="n">
-        <v>-20.6</v>
+        <v>-21.1</v>
       </c>
       <c r="I124" t="n">
         <v>396.9</v>
       </c>
       <c r="J124" t="n">
-        <v>-3.6</v>
+        <v>-4.2</v>
       </c>
       <c r="K124" t="n">
-        <v>555</v>
+        <v>552</v>
       </c>
       <c r="L124" t="n">
-        <v>45</v>
+        <v>45.1</v>
       </c>
       <c r="M124" t="n">
-        <v>1.6</v>
+        <v>1.1</v>
       </c>
       <c r="N124" t="n">
         <v>558.1</v>
       </c>
       <c r="O124" t="n">
-        <v>-0.6</v>
+        <v>-1.1</v>
       </c>
       <c r="P124" t="n">
-        <v>1838.9</v>
+        <v>1834.1</v>
       </c>
       <c r="Q124" t="n">
-        <v>0.5</v>
+        <v>0.2</v>
       </c>
       <c r="R124" t="n">
         <v>1863.3</v>
       </c>
       <c r="S124" t="n">
-        <v>-1.3</v>
+        <v>-1.6</v>
       </c>
       <c r="T124" t="n">
-        <v>2159.2</v>
+        <v>2165.4</v>
       </c>
       <c r="U124" t="n">
-        <v>17.4</v>
+        <v>18.1</v>
       </c>
       <c r="V124" t="n">
         <v>2155.7</v>
       </c>
       <c r="W124" t="n">
-        <v>0.2</v>
+        <v>0.4</v>
       </c>
       <c r="X124" t="n">
-        <v>2385.9</v>
+        <v>2388.5</v>
       </c>
       <c r="Y124" t="n">
-        <v>10.5</v>
+        <v>10.3</v>
       </c>
       <c r="Z124" t="n">
         <v>2405.8</v>
       </c>
       <c r="AA124" t="n">
-        <v>-0.8</v>
+        <v>-0.7</v>
       </c>
       <c r="AB124" t="n">
         <v>82500</v>
@@ -13742,40 +13742,40 @@
         </is>
       </c>
       <c r="F134" t="n">
-        <v>20650.6</v>
+        <v>20523</v>
       </c>
       <c r="G134" t="n">
-        <v>-16.6</v>
+        <v>-17.1</v>
       </c>
       <c r="H134" t="n">
-        <v>5.7</v>
+        <v>5</v>
       </c>
       <c r="I134" t="n">
         <v>20703</v>
       </c>
       <c r="J134" t="n">
-        <v>-0.3</v>
+        <v>-0.9</v>
       </c>
       <c r="K134" t="n">
-        <v>11546.4</v>
+        <v>11517</v>
       </c>
       <c r="L134" t="n">
-        <v>-44.1</v>
+        <v>-43.9</v>
       </c>
       <c r="M134" t="n">
-        <v>4</v>
+        <v>3.7</v>
       </c>
       <c r="N134" t="n">
         <v>11584</v>
       </c>
       <c r="O134" t="n">
-        <v>-0.3</v>
+        <v>-0.6</v>
       </c>
       <c r="P134" t="n">
-        <v>78789.8</v>
+        <v>78747.2</v>
       </c>
       <c r="Q134" t="n">
-        <v>12.2</v>
+        <v>12.1</v>
       </c>
       <c r="R134" t="n">
         <v>78928.60000000001</v>
@@ -13784,28 +13784,28 @@
         <v>-0.2</v>
       </c>
       <c r="T134" t="n">
-        <v>82922.39999999999</v>
+        <v>82960.89999999999</v>
       </c>
       <c r="U134" t="n">
-        <v>5.2</v>
+        <v>5.4</v>
       </c>
       <c r="V134" t="n">
         <v>82823.2</v>
       </c>
       <c r="W134" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="X134" t="n">
-        <v>87020.2</v>
+        <v>87303.10000000001</v>
       </c>
       <c r="Y134" t="n">
-        <v>4.9</v>
+        <v>5.2</v>
       </c>
       <c r="Z134" t="n">
         <v>86770.8</v>
       </c>
       <c r="AA134" t="n">
-        <v>0.3</v>
+        <v>0.6</v>
       </c>
       <c r="AB134" t="n">
         <v>88000</v>
@@ -14120,70 +14120,70 @@
         </is>
       </c>
       <c r="F138" t="n">
-        <v>643.6</v>
+        <v>635.6</v>
       </c>
       <c r="G138" t="n">
-        <v>3.7</v>
+        <v>2.5</v>
       </c>
       <c r="H138" t="n">
-        <v>51.2</v>
+        <v>49.3</v>
       </c>
       <c r="I138" t="n">
         <v>657.7</v>
       </c>
       <c r="J138" t="n">
-        <v>-2.1</v>
+        <v>-3.4</v>
       </c>
       <c r="K138" t="n">
-        <v>704.7</v>
+        <v>709.7</v>
       </c>
       <c r="L138" t="n">
-        <v>9.5</v>
+        <v>11.7</v>
       </c>
       <c r="M138" t="n">
-        <v>34.6</v>
+        <v>35.5</v>
       </c>
       <c r="N138" t="n">
         <v>707.5</v>
       </c>
       <c r="O138" t="n">
-        <v>-0.4</v>
+        <v>0.3</v>
       </c>
       <c r="P138" t="n">
-        <v>2525.2</v>
+        <v>2522.2</v>
       </c>
       <c r="Q138" t="n">
-        <v>41.4</v>
+        <v>41.2</v>
       </c>
       <c r="R138" t="n">
         <v>2541.9</v>
       </c>
       <c r="S138" t="n">
-        <v>-0.7</v>
+        <v>-0.8</v>
       </c>
       <c r="T138" t="n">
-        <v>3389</v>
+        <v>3402</v>
       </c>
       <c r="U138" t="n">
-        <v>34.2</v>
+        <v>34.9</v>
       </c>
       <c r="V138" t="n">
         <v>3404.3</v>
       </c>
       <c r="W138" t="n">
-        <v>-0.4</v>
+        <v>-0.1</v>
       </c>
       <c r="X138" t="n">
-        <v>4410.4</v>
+        <v>4412.4</v>
       </c>
       <c r="Y138" t="n">
-        <v>30.1</v>
+        <v>29.7</v>
       </c>
       <c r="Z138" t="n">
         <v>4411.6</v>
       </c>
       <c r="AA138" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AB138" t="n">
         <v>162700</v>
@@ -15006,55 +15006,55 @@
         <v>0</v>
       </c>
       <c r="K147" t="n">
-        <v>5862.8</v>
+        <v>5902</v>
       </c>
       <c r="L147" t="n">
-        <v>15</v>
+        <v>15.8</v>
       </c>
       <c r="M147" t="n">
-        <v>23.4</v>
+        <v>24.2</v>
       </c>
       <c r="N147" t="n">
         <v>5862.8</v>
       </c>
       <c r="O147" t="n">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="P147" t="n">
-        <v>18617.5</v>
+        <v>18697.7</v>
       </c>
       <c r="Q147" t="n">
-        <v>59.3</v>
+        <v>60</v>
       </c>
       <c r="R147" t="n">
         <v>18617.5</v>
       </c>
       <c r="S147" t="n">
-        <v>0</v>
+        <v>0.4</v>
       </c>
       <c r="T147" t="n">
-        <v>22916.2</v>
+        <v>23047.7</v>
       </c>
       <c r="U147" t="n">
-        <v>23.1</v>
+        <v>23.3</v>
       </c>
       <c r="V147" t="n">
         <v>22916.2</v>
       </c>
       <c r="W147" t="n">
-        <v>0</v>
+        <v>0.6</v>
       </c>
       <c r="X147" t="n">
-        <v>25807.6</v>
+        <v>25964.3</v>
       </c>
       <c r="Y147" t="n">
-        <v>12.6</v>
+        <v>12.7</v>
       </c>
       <c r="Z147" t="n">
         <v>25807.6</v>
       </c>
       <c r="AA147" t="n">
-        <v>0</v>
+        <v>0.6</v>
       </c>
       <c r="AB147" t="n">
         <v>192600</v>
@@ -15924,19 +15924,19 @@
         </is>
       </c>
       <c r="F157" t="n">
-        <v>113</v>
+        <v>106</v>
       </c>
       <c r="G157" t="n">
-        <v>11.9</v>
+        <v>5</v>
       </c>
       <c r="H157" t="n">
-        <v>606.2</v>
+        <v>562.5</v>
       </c>
       <c r="I157" t="n">
         <v>117</v>
       </c>
       <c r="J157" t="n">
-        <v>-3.4</v>
+        <v>-9.4</v>
       </c>
       <c r="AB157" t="n">
         <v>11140</v>
@@ -16799,25 +16799,25 @@
         </is>
       </c>
       <c r="F167" t="n">
-        <v>896.8</v>
+        <v>480.8</v>
       </c>
       <c r="G167" t="n">
-        <v>-85.7</v>
+        <v>-92.3</v>
       </c>
       <c r="H167" t="n">
-        <v>-74.7</v>
+        <v>-86.5</v>
       </c>
       <c r="I167" t="n">
         <v>1615.2</v>
       </c>
       <c r="J167" t="n">
-        <v>-44.5</v>
+        <v>-70.2</v>
       </c>
       <c r="K167" t="n">
         <v>1161.2</v>
       </c>
       <c r="L167" t="n">
-        <v>29.5</v>
+        <v>141.5</v>
       </c>
       <c r="M167" t="n">
         <v>-35.6</v>
@@ -16829,40 +16829,40 @@
         <v>-8.1</v>
       </c>
       <c r="P167" t="n">
-        <v>9091.299999999999</v>
+        <v>8850.200000000001</v>
       </c>
       <c r="Q167" t="n">
-        <v>-20.8</v>
+        <v>-22.9</v>
       </c>
       <c r="R167" t="n">
         <v>9436.9</v>
       </c>
       <c r="S167" t="n">
-        <v>-3.7</v>
+        <v>-6.2</v>
       </c>
       <c r="T167" t="n">
-        <v>10057.6</v>
+        <v>10098.7</v>
       </c>
       <c r="U167" t="n">
-        <v>10.6</v>
+        <v>14.1</v>
       </c>
       <c r="V167" t="n">
         <v>10008.7</v>
       </c>
       <c r="W167" t="n">
-        <v>0.5</v>
+        <v>0.9</v>
       </c>
       <c r="X167" t="n">
-        <v>10740</v>
+        <v>10821.1</v>
       </c>
       <c r="Y167" t="n">
-        <v>6.8</v>
+        <v>7.2</v>
       </c>
       <c r="Z167" t="n">
         <v>10693.3</v>
       </c>
       <c r="AA167" t="n">
-        <v>0.4</v>
+        <v>1.2</v>
       </c>
       <c r="AB167" t="n">
         <v>3985</v>
@@ -16901,70 +16901,70 @@
         </is>
       </c>
       <c r="F168" t="n">
-        <v>918.4</v>
+        <v>918</v>
       </c>
       <c r="G168" t="n">
         <v>8.5</v>
       </c>
       <c r="H168" t="n">
-        <v>3.2</v>
+        <v>3.1</v>
       </c>
       <c r="I168" t="n">
         <v>924.1</v>
       </c>
       <c r="J168" t="n">
-        <v>-0.6</v>
+        <v>-0.7</v>
       </c>
       <c r="K168" t="n">
-        <v>895</v>
+        <v>888.6</v>
       </c>
       <c r="L168" t="n">
-        <v>-2.5</v>
+        <v>-3.2</v>
       </c>
       <c r="M168" t="n">
-        <v>12.9</v>
+        <v>12.1</v>
       </c>
       <c r="N168" t="n">
         <v>895.3</v>
       </c>
       <c r="O168" t="n">
-        <v>-0</v>
+        <v>-0.7</v>
       </c>
       <c r="P168" t="n">
-        <v>3496.6</v>
+        <v>3492.1</v>
       </c>
       <c r="Q168" t="n">
-        <v>11.9</v>
+        <v>11.7</v>
       </c>
       <c r="R168" t="n">
         <v>3505.9</v>
       </c>
       <c r="S168" t="n">
-        <v>-0.3</v>
+        <v>-0.4</v>
       </c>
       <c r="T168" t="n">
-        <v>3822.4</v>
+        <v>3799</v>
       </c>
       <c r="U168" t="n">
-        <v>9.300000000000001</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="V168" t="n">
         <v>3833</v>
       </c>
       <c r="W168" t="n">
-        <v>-0.3</v>
+        <v>-0.9</v>
       </c>
       <c r="X168" t="n">
-        <v>4171.8</v>
+        <v>4141.6</v>
       </c>
       <c r="Y168" t="n">
-        <v>9.1</v>
+        <v>9</v>
       </c>
       <c r="Z168" t="n">
         <v>4151.2</v>
       </c>
       <c r="AA168" t="n">
-        <v>0.5</v>
+        <v>-0.2</v>
       </c>
       <c r="AB168" t="n">
         <v>50300</v>
@@ -18176,37 +18176,37 @@
         </is>
       </c>
       <c r="F182" t="n">
-        <v>25452.2</v>
+        <v>25429.3</v>
       </c>
       <c r="G182" t="n">
-        <v>-6.2</v>
+        <v>-6.3</v>
       </c>
       <c r="H182" t="n">
-        <v>9</v>
+        <v>8.9</v>
       </c>
       <c r="I182" t="n">
         <v>25528.5</v>
       </c>
       <c r="J182" t="n">
-        <v>-0.3</v>
+        <v>-0.4</v>
       </c>
       <c r="K182" t="n">
-        <v>14423.3</v>
+        <v>14413.6</v>
       </c>
       <c r="L182" t="n">
         <v>-43.3</v>
       </c>
       <c r="M182" t="n">
-        <v>-17.9</v>
+        <v>-18</v>
       </c>
       <c r="N182" t="n">
         <v>14442.7</v>
       </c>
       <c r="O182" t="n">
-        <v>-0.1</v>
+        <v>-0.2</v>
       </c>
       <c r="P182" t="n">
-        <v>94139.5</v>
+        <v>94107.7</v>
       </c>
       <c r="Q182" t="n">
         <v>10.5</v>
@@ -18215,10 +18215,10 @@
         <v>94352.39999999999</v>
       </c>
       <c r="S182" t="n">
-        <v>-0.2</v>
+        <v>-0.3</v>
       </c>
       <c r="T182" t="n">
-        <v>95973</v>
+        <v>95857.3</v>
       </c>
       <c r="U182" t="n">
         <v>1.9</v>
@@ -18227,10 +18227,10 @@
         <v>96183.8</v>
       </c>
       <c r="W182" t="n">
-        <v>-0.2</v>
+        <v>-0.3</v>
       </c>
       <c r="X182" t="n">
-        <v>99679.89999999999</v>
+        <v>99579.3</v>
       </c>
       <c r="Y182" t="n">
         <v>3.9</v>
@@ -18239,7 +18239,7 @@
         <v>99708.7</v>
       </c>
       <c r="AA182" t="n">
-        <v>-0</v>
+        <v>-0.1</v>
       </c>
       <c r="AB182" t="n">
         <v>153000</v>
@@ -18384,70 +18384,70 @@
         </is>
       </c>
       <c r="F184" t="n">
-        <v>2072.9</v>
+        <v>2051.7</v>
       </c>
       <c r="G184" t="n">
-        <v>18.1</v>
+        <v>16.9</v>
       </c>
       <c r="H184" t="n">
-        <v>14.4</v>
+        <v>13.2</v>
       </c>
       <c r="I184" t="n">
         <v>2072.9</v>
       </c>
       <c r="J184" t="n">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="K184" t="n">
-        <v>1240.1</v>
+        <v>1226.8</v>
       </c>
       <c r="L184" t="n">
         <v>-40.2</v>
       </c>
       <c r="M184" t="n">
-        <v>17.9</v>
+        <v>16.6</v>
       </c>
       <c r="N184" t="n">
         <v>1240.1</v>
       </c>
       <c r="O184" t="n">
-        <v>0</v>
+        <v>-1.1</v>
       </c>
       <c r="P184" t="n">
-        <v>6330.3</v>
+        <v>6266.7</v>
       </c>
       <c r="Q184" t="n">
-        <v>23.1</v>
+        <v>21.8</v>
       </c>
       <c r="R184" t="n">
         <v>6330.3</v>
       </c>
       <c r="S184" t="n">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="T184" t="n">
-        <v>6940.1</v>
+        <v>6826.7</v>
       </c>
       <c r="U184" t="n">
-        <v>9.6</v>
+        <v>8.9</v>
       </c>
       <c r="V184" t="n">
         <v>6940.1</v>
       </c>
       <c r="W184" t="n">
-        <v>0</v>
+        <v>-1.6</v>
       </c>
       <c r="X184" t="n">
-        <v>7645.2</v>
+        <v>7376</v>
       </c>
       <c r="Y184" t="n">
-        <v>10.2</v>
+        <v>8</v>
       </c>
       <c r="Z184" t="n">
         <v>7645.2</v>
       </c>
       <c r="AA184" t="n">
-        <v>0</v>
+        <v>-3.5</v>
       </c>
       <c r="AB184" t="n">
         <v>69700</v>
@@ -18486,70 +18486,70 @@
         </is>
       </c>
       <c r="F185" t="n">
-        <v>826.7</v>
+        <v>815.9</v>
       </c>
       <c r="G185" t="n">
-        <v>-3.9</v>
+        <v>-5.2</v>
       </c>
       <c r="H185" t="n">
-        <v>25.8</v>
+        <v>24.2</v>
       </c>
       <c r="I185" t="n">
         <v>826.7</v>
       </c>
       <c r="J185" t="n">
-        <v>0</v>
+        <v>-1.3</v>
       </c>
       <c r="K185" t="n">
-        <v>606.8</v>
+        <v>617.3</v>
       </c>
       <c r="L185" t="n">
-        <v>-26.6</v>
+        <v>-24.3</v>
       </c>
       <c r="M185" t="n">
-        <v>-13.5</v>
+        <v>-12</v>
       </c>
       <c r="N185" t="n">
         <v>606.8</v>
       </c>
       <c r="O185" t="n">
-        <v>0</v>
+        <v>1.7</v>
       </c>
       <c r="P185" t="n">
-        <v>3035.4</v>
+        <v>3034.2</v>
       </c>
       <c r="Q185" t="n">
-        <v>-5.2</v>
+        <v>-5.3</v>
       </c>
       <c r="R185" t="n">
         <v>3035.4</v>
       </c>
       <c r="S185" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="T185" t="n">
-        <v>3365.3</v>
+        <v>3330.7</v>
       </c>
       <c r="U185" t="n">
-        <v>10.9</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="V185" t="n">
         <v>3365.3</v>
       </c>
       <c r="W185" t="n">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="X185" t="n">
-        <v>2642.8</v>
+        <v>2582.5</v>
       </c>
       <c r="Y185" t="n">
-        <v>-21.5</v>
+        <v>-22.5</v>
       </c>
       <c r="Z185" t="n">
         <v>2642.8</v>
       </c>
       <c r="AA185" t="n">
-        <v>0</v>
+        <v>-2.3</v>
       </c>
       <c r="AB185" t="n">
         <v>43450</v>
@@ -21207,10 +21207,10 @@
         <v>-3.2</v>
       </c>
       <c r="P212" t="n">
-        <v>24577.9</v>
+        <v>24562</v>
       </c>
       <c r="Q212" t="n">
-        <v>18.8</v>
+        <v>18.7</v>
       </c>
       <c r="R212" t="n">
         <v>24521.1</v>
@@ -21219,28 +21219,28 @@
         <v>0.2</v>
       </c>
       <c r="T212" t="n">
-        <v>28826.5</v>
+        <v>28728.2</v>
       </c>
       <c r="U212" t="n">
-        <v>17.3</v>
+        <v>17</v>
       </c>
       <c r="V212" t="n">
         <v>28668.1</v>
       </c>
       <c r="W212" t="n">
-        <v>0.6</v>
+        <v>0.2</v>
       </c>
       <c r="X212" t="n">
-        <v>31334.8</v>
+        <v>31258.1</v>
       </c>
       <c r="Y212" t="n">
-        <v>8.699999999999999</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="Z212" t="n">
         <v>30906.4</v>
       </c>
       <c r="AA212" t="n">
-        <v>1.4</v>
+        <v>1.1</v>
       </c>
       <c r="AB212" t="n">
         <v>1460000</v>
@@ -21279,19 +21279,19 @@
         </is>
       </c>
       <c r="F213" t="n">
-        <v>474</v>
+        <v>460</v>
       </c>
       <c r="G213" t="n">
-        <v>8</v>
+        <v>4.8</v>
       </c>
       <c r="H213" t="n">
-        <v>26.1</v>
+        <v>22.3</v>
       </c>
       <c r="I213" t="n">
         <v>492</v>
       </c>
       <c r="J213" t="n">
-        <v>-3.7</v>
+        <v>-6.5</v>
       </c>
       <c r="AB213" t="n">
         <v>27500</v>
@@ -21534,70 +21534,70 @@
         </is>
       </c>
       <c r="F216" t="n">
-        <v>855.2</v>
+        <v>851.5</v>
       </c>
       <c r="G216" t="n">
-        <v>36</v>
+        <v>35.4</v>
       </c>
       <c r="H216" t="n">
-        <v>590.2</v>
+        <v>587.2</v>
       </c>
       <c r="I216" t="n">
         <v>862.9</v>
       </c>
       <c r="J216" t="n">
-        <v>-0.9</v>
+        <v>-1.3</v>
       </c>
       <c r="K216" t="n">
-        <v>952.8</v>
+        <v>954.2</v>
       </c>
       <c r="L216" t="n">
-        <v>11.4</v>
+        <v>12.1</v>
       </c>
       <c r="M216" t="n">
-        <v>828.7</v>
+        <v>830</v>
       </c>
       <c r="N216" t="n">
         <v>965.4</v>
       </c>
       <c r="O216" t="n">
-        <v>-1.3</v>
+        <v>-1.2</v>
       </c>
       <c r="P216" t="n">
-        <v>2573.1</v>
+        <v>2570.8</v>
       </c>
       <c r="Q216" t="n">
-        <v>2067.7</v>
+        <v>2065.8</v>
       </c>
       <c r="R216" t="n">
         <v>2593.4</v>
       </c>
       <c r="S216" t="n">
-        <v>-0.8</v>
+        <v>-0.9</v>
       </c>
       <c r="T216" t="n">
-        <v>4368.5</v>
+        <v>4397.2</v>
       </c>
       <c r="U216" t="n">
-        <v>69.8</v>
+        <v>71</v>
       </c>
       <c r="V216" t="n">
         <v>4386.8</v>
       </c>
       <c r="W216" t="n">
-        <v>-0.4</v>
+        <v>0.2</v>
       </c>
       <c r="X216" t="n">
-        <v>5696.2</v>
+        <v>5728.2</v>
       </c>
       <c r="Y216" t="n">
-        <v>30.4</v>
+        <v>30.3</v>
       </c>
       <c r="Z216" t="n">
         <v>5684</v>
       </c>
       <c r="AA216" t="n">
-        <v>0.2</v>
+        <v>0.8</v>
       </c>
       <c r="AB216" t="n">
         <v>111400</v>
@@ -21840,70 +21840,70 @@
         </is>
       </c>
       <c r="F219" t="n">
-        <v>1672.4</v>
+        <v>1760.5</v>
       </c>
       <c r="G219" t="n">
-        <v>-42.1</v>
+        <v>-39.1</v>
       </c>
       <c r="H219" t="n">
-        <v>21.3</v>
+        <v>27.7</v>
       </c>
       <c r="I219" t="n">
         <v>1672.4</v>
       </c>
       <c r="J219" t="n">
-        <v>0</v>
+        <v>5.3</v>
       </c>
       <c r="K219" t="n">
-        <v>1605</v>
+        <v>1673.3</v>
       </c>
       <c r="L219" t="n">
-        <v>-4</v>
+        <v>-5</v>
       </c>
       <c r="M219" t="n">
-        <v>8.199999999999999</v>
+        <v>12.8</v>
       </c>
       <c r="N219" t="n">
         <v>1605</v>
       </c>
       <c r="O219" t="n">
-        <v>0</v>
+        <v>4.3</v>
       </c>
       <c r="P219" t="n">
-        <v>8312.5</v>
+        <v>8434.200000000001</v>
       </c>
       <c r="Q219" t="n">
-        <v>21.2</v>
+        <v>22.9</v>
       </c>
       <c r="R219" t="n">
         <v>8312.5</v>
       </c>
       <c r="S219" t="n">
-        <v>0</v>
+        <v>1.5</v>
       </c>
       <c r="T219" t="n">
-        <v>8512.700000000001</v>
+        <v>8459.6</v>
       </c>
       <c r="U219" t="n">
-        <v>2.4</v>
+        <v>0.3</v>
       </c>
       <c r="V219" t="n">
         <v>8512.700000000001</v>
       </c>
       <c r="W219" t="n">
-        <v>0</v>
+        <v>-0.6</v>
       </c>
       <c r="X219" t="n">
-        <v>9544.5</v>
+        <v>9649.6</v>
       </c>
       <c r="Y219" t="n">
-        <v>12.1</v>
+        <v>14.1</v>
       </c>
       <c r="Z219" t="n">
         <v>9544.5</v>
       </c>
       <c r="AA219" t="n">
-        <v>0</v>
+        <v>1.1</v>
       </c>
       <c r="AB219" t="n">
         <v>49000</v>
@@ -23068,64 +23068,64 @@
         </is>
       </c>
       <c r="F231" t="n">
-        <v>1542.6</v>
+        <v>1540.5</v>
       </c>
       <c r="G231" t="n">
-        <v>16.4</v>
+        <v>16.2</v>
       </c>
       <c r="H231" t="n">
-        <v>11.9</v>
+        <v>11.7</v>
       </c>
       <c r="I231" t="n">
         <v>1548.1</v>
       </c>
       <c r="J231" t="n">
-        <v>-0.4</v>
+        <v>-0.5</v>
       </c>
       <c r="K231" t="n">
-        <v>1840.6</v>
+        <v>1838.8</v>
       </c>
       <c r="L231" t="n">
-        <v>19.3</v>
+        <v>19.4</v>
       </c>
       <c r="M231" t="n">
-        <v>9.800000000000001</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="N231" t="n">
         <v>1839.4</v>
       </c>
       <c r="O231" t="n">
-        <v>0.1</v>
+        <v>-0</v>
       </c>
       <c r="P231" t="n">
-        <v>6365.1</v>
+        <v>6361.1</v>
       </c>
       <c r="Q231" t="n">
-        <v>14</v>
+        <v>13.9</v>
       </c>
       <c r="R231" t="n">
         <v>6372.8</v>
       </c>
       <c r="S231" t="n">
-        <v>-0.1</v>
+        <v>-0.2</v>
       </c>
       <c r="T231" t="n">
-        <v>6910.3</v>
+        <v>6895.9</v>
       </c>
       <c r="U231" t="n">
-        <v>8.6</v>
+        <v>8.4</v>
       </c>
       <c r="V231" t="n">
         <v>6937.7</v>
       </c>
       <c r="W231" t="n">
-        <v>-0.4</v>
+        <v>-0.6</v>
       </c>
       <c r="X231" t="n">
         <v>7433</v>
       </c>
       <c r="Y231" t="n">
-        <v>7.6</v>
+        <v>7.8</v>
       </c>
       <c r="Z231" t="n">
         <v>7503.3</v>
@@ -23503,7 +23503,7 @@
         </is>
       </c>
       <c r="F236" t="n">
-        <v>863.1</v>
+        <v>863.3</v>
       </c>
       <c r="G236" t="n">
         <v>33.4</v>
@@ -23518,10 +23518,10 @@
         <v>-0.2</v>
       </c>
       <c r="K236" t="n">
-        <v>281.1</v>
+        <v>281</v>
       </c>
       <c r="L236" t="n">
-        <v>-67.40000000000001</v>
+        <v>-67.5</v>
       </c>
       <c r="M236" t="inlineStr">
         <is>
@@ -23535,7 +23535,7 @@
         <v>0.2</v>
       </c>
       <c r="P236" t="n">
-        <v>2149.1</v>
+        <v>2149.2</v>
       </c>
       <c r="Q236" t="n">
         <v>96.2</v>
@@ -23547,22 +23547,22 @@
         <v>0</v>
       </c>
       <c r="T236" t="n">
-        <v>2410.9</v>
+        <v>2408.5</v>
       </c>
       <c r="U236" t="n">
-        <v>12.2</v>
+        <v>12.1</v>
       </c>
       <c r="V236" t="n">
         <v>2409.4</v>
       </c>
       <c r="W236" t="n">
-        <v>0.1</v>
+        <v>-0</v>
       </c>
       <c r="X236" t="n">
         <v>2673.3</v>
       </c>
       <c r="Y236" t="n">
-        <v>10.9</v>
+        <v>11</v>
       </c>
       <c r="Z236" t="n">
         <v>2667.2</v>
@@ -24403,10 +24403,10 @@
         </is>
       </c>
       <c r="F245" t="n">
-        <v>237.2</v>
+        <v>229.3</v>
       </c>
       <c r="G245" t="n">
-        <v>-32.1</v>
+        <v>-34.4</v>
       </c>
       <c r="H245" t="inlineStr">
         <is>
@@ -24417,52 +24417,52 @@
         <v>232.7</v>
       </c>
       <c r="J245" t="n">
-        <v>1.9</v>
+        <v>-1.5</v>
       </c>
       <c r="K245" t="n">
-        <v>302</v>
+        <v>293.3</v>
       </c>
       <c r="L245" t="n">
-        <v>27.3</v>
+        <v>27.9</v>
       </c>
       <c r="M245" t="n">
-        <v>264.7</v>
+        <v>254.2</v>
       </c>
       <c r="N245" t="n">
         <v>285</v>
       </c>
       <c r="O245" t="n">
-        <v>6</v>
+        <v>2.9</v>
       </c>
       <c r="P245" t="n">
-        <v>1130.4</v>
+        <v>1113.7</v>
       </c>
       <c r="Q245" t="n">
-        <v>127.9</v>
+        <v>124.5</v>
       </c>
       <c r="R245" t="n">
         <v>1098.8</v>
       </c>
       <c r="S245" t="n">
-        <v>2.9</v>
+        <v>1.4</v>
       </c>
       <c r="T245" t="n">
-        <v>1374.2</v>
+        <v>1325.2</v>
       </c>
       <c r="U245" t="n">
-        <v>21.6</v>
+        <v>19</v>
       </c>
       <c r="V245" t="n">
         <v>1316.8</v>
       </c>
       <c r="W245" t="n">
-        <v>4.4</v>
+        <v>0.6</v>
       </c>
       <c r="X245" t="n">
         <v>1468.2</v>
       </c>
       <c r="Y245" t="n">
-        <v>6.8</v>
+        <v>10.8</v>
       </c>
       <c r="Z245" t="n">
         <v>1468.2</v>
@@ -24815,70 +24815,70 @@
         </is>
       </c>
       <c r="F249" t="n">
-        <v>551.5</v>
+        <v>553.2</v>
       </c>
       <c r="G249" t="n">
-        <v>9.699999999999999</v>
+        <v>10.1</v>
       </c>
       <c r="H249" t="n">
-        <v>135.7</v>
+        <v>136.4</v>
       </c>
       <c r="I249" t="n">
         <v>536.8</v>
       </c>
       <c r="J249" t="n">
-        <v>2.7</v>
+        <v>3.1</v>
       </c>
       <c r="K249" t="n">
-        <v>424.5</v>
+        <v>437.6</v>
       </c>
       <c r="L249" t="n">
-        <v>-23</v>
+        <v>-20.9</v>
       </c>
       <c r="M249" t="n">
-        <v>93.8</v>
+        <v>99.8</v>
       </c>
       <c r="N249" t="n">
         <v>403.5</v>
       </c>
       <c r="O249" t="n">
-        <v>5.2</v>
+        <v>8.5</v>
       </c>
       <c r="P249" t="n">
-        <v>1951</v>
+        <v>1966.8</v>
       </c>
       <c r="Q249" t="n">
-        <v>120.5</v>
+        <v>122.3</v>
       </c>
       <c r="R249" t="n">
         <v>1915</v>
       </c>
       <c r="S249" t="n">
-        <v>1.9</v>
+        <v>2.7</v>
       </c>
       <c r="T249" t="n">
-        <v>2384</v>
+        <v>2393.2</v>
       </c>
       <c r="U249" t="n">
-        <v>22.2</v>
+        <v>21.7</v>
       </c>
       <c r="V249" t="n">
         <v>2353.2</v>
       </c>
       <c r="W249" t="n">
-        <v>1.3</v>
+        <v>1.7</v>
       </c>
       <c r="X249" t="n">
-        <v>2465.8</v>
+        <v>2568.6</v>
       </c>
       <c r="Y249" t="n">
-        <v>3.4</v>
+        <v>7.3</v>
       </c>
       <c r="Z249" t="n">
         <v>2443.2</v>
       </c>
       <c r="AA249" t="n">
-        <v>0.9</v>
+        <v>5.1</v>
       </c>
       <c r="AB249" t="n">
         <v>115900</v>
@@ -25342,25 +25342,25 @@
         <v>0.5</v>
       </c>
       <c r="K254" t="n">
-        <v>800.4</v>
+        <v>800.8</v>
       </c>
       <c r="L254" t="n">
         <v>4.3</v>
       </c>
       <c r="M254" t="n">
-        <v>176.5</v>
+        <v>176.6</v>
       </c>
       <c r="N254" t="n">
         <v>794.6</v>
       </c>
       <c r="O254" t="n">
-        <v>0.7</v>
+        <v>0.8</v>
       </c>
       <c r="P254" t="n">
-        <v>2783.5</v>
+        <v>2784</v>
       </c>
       <c r="Q254" t="n">
-        <v>467.4</v>
+        <v>467.5</v>
       </c>
       <c r="R254" t="n">
         <v>2775</v>
@@ -25369,28 +25369,28 @@
         <v>0.3</v>
       </c>
       <c r="T254" t="n">
-        <v>4150.5</v>
+        <v>4174.2</v>
       </c>
       <c r="U254" t="n">
-        <v>49.1</v>
+        <v>49.9</v>
       </c>
       <c r="V254" t="n">
         <v>4106.6</v>
       </c>
       <c r="W254" t="n">
-        <v>1.1</v>
+        <v>1.6</v>
       </c>
       <c r="X254" t="n">
-        <v>5164.4</v>
+        <v>5186.1</v>
       </c>
       <c r="Y254" t="n">
-        <v>24.4</v>
+        <v>24.2</v>
       </c>
       <c r="Z254" t="n">
         <v>5127.8</v>
       </c>
       <c r="AA254" t="n">
-        <v>0.7</v>
+        <v>1.1</v>
       </c>
       <c r="AB254" t="n">
         <v>122700</v>
@@ -26057,70 +26057,70 @@
         </is>
       </c>
       <c r="F261" t="n">
-        <v>1310.8</v>
+        <v>1286.1</v>
       </c>
       <c r="G261" t="n">
-        <v>51.5</v>
+        <v>48.7</v>
       </c>
       <c r="H261" t="n">
-        <v>2.4</v>
+        <v>0.5</v>
       </c>
       <c r="I261" t="n">
         <v>1335.8</v>
       </c>
       <c r="J261" t="n">
-        <v>-1.9</v>
+        <v>-3.7</v>
       </c>
       <c r="K261" t="n">
-        <v>1477.2</v>
+        <v>1468</v>
       </c>
       <c r="L261" t="n">
-        <v>12.7</v>
+        <v>14.1</v>
       </c>
       <c r="M261" t="n">
-        <v>11.1</v>
+        <v>10.5</v>
       </c>
       <c r="N261" t="n">
         <v>1491</v>
       </c>
       <c r="O261" t="n">
-        <v>-0.9</v>
+        <v>-1.5</v>
       </c>
       <c r="P261" t="n">
-        <v>5205</v>
+        <v>5152.7</v>
       </c>
       <c r="Q261" t="n">
-        <v>11.1</v>
+        <v>10</v>
       </c>
       <c r="R261" t="n">
         <v>5266.2</v>
       </c>
       <c r="S261" t="n">
-        <v>-1.2</v>
+        <v>-2.2</v>
       </c>
       <c r="T261" t="n">
-        <v>5622</v>
+        <v>5549.7</v>
       </c>
       <c r="U261" t="n">
-        <v>8</v>
+        <v>7.7</v>
       </c>
       <c r="V261" t="n">
         <v>5678.2</v>
       </c>
       <c r="W261" t="n">
-        <v>-1</v>
+        <v>-2.3</v>
       </c>
       <c r="X261" t="n">
-        <v>6128.6</v>
+        <v>5988.3</v>
       </c>
       <c r="Y261" t="n">
-        <v>9</v>
+        <v>7.9</v>
       </c>
       <c r="Z261" t="n">
         <v>6195.7</v>
       </c>
       <c r="AA261" t="n">
-        <v>-1.1</v>
+        <v>-3.3</v>
       </c>
       <c r="AB261" t="n">
         <v>63100</v>
@@ -26781,10 +26781,10 @@
         </is>
       </c>
       <c r="F270" t="n">
-        <v>433</v>
+        <v>326</v>
       </c>
       <c r="G270" t="n">
-        <v>0.1</v>
+        <v>-24.6</v>
       </c>
       <c r="H270" t="inlineStr">
         <is>
@@ -26795,58 +26795,58 @@
         <v>433</v>
       </c>
       <c r="J270" t="n">
-        <v>0</v>
+        <v>-24.7</v>
       </c>
       <c r="K270" t="n">
-        <v>392.5</v>
+        <v>285</v>
       </c>
       <c r="L270" t="n">
-        <v>-9.4</v>
+        <v>-12.6</v>
       </c>
       <c r="M270" t="n">
-        <v>1296.8</v>
+        <v>914.2</v>
       </c>
       <c r="N270" t="n">
         <v>392.5</v>
       </c>
       <c r="O270" t="n">
-        <v>0</v>
+        <v>-27.4</v>
       </c>
       <c r="P270" t="n">
-        <v>1440.7</v>
+        <v>1286</v>
       </c>
       <c r="Q270" t="n">
-        <v>32643.2</v>
+        <v>29127.3</v>
       </c>
       <c r="R270" t="n">
         <v>1536</v>
       </c>
       <c r="S270" t="n">
-        <v>-6.2</v>
+        <v>-16.3</v>
       </c>
       <c r="T270" t="n">
-        <v>1692.3</v>
+        <v>1478.5</v>
       </c>
       <c r="U270" t="n">
-        <v>17.5</v>
+        <v>15</v>
       </c>
       <c r="V270" t="n">
         <v>1758.5</v>
       </c>
       <c r="W270" t="n">
-        <v>-3.8</v>
+        <v>-15.9</v>
       </c>
       <c r="X270" t="n">
-        <v>1726.7</v>
+        <v>1505</v>
       </c>
       <c r="Y270" t="n">
-        <v>2</v>
+        <v>1.8</v>
       </c>
       <c r="Z270" t="n">
         <v>1775</v>
       </c>
       <c r="AA270" t="n">
-        <v>-2.7</v>
+        <v>-15.2</v>
       </c>
       <c r="AB270" t="n">
         <v>59500</v>
@@ -27040,49 +27040,49 @@
         </is>
       </c>
       <c r="F273" t="n">
-        <v>257.7</v>
+        <v>255.4</v>
       </c>
       <c r="G273" t="n">
-        <v>-8.4</v>
+        <v>-9.199999999999999</v>
       </c>
       <c r="H273" t="n">
-        <v>-48</v>
+        <v>-48.5</v>
       </c>
       <c r="I273" t="n">
         <v>254</v>
       </c>
       <c r="J273" t="n">
-        <v>1.5</v>
+        <v>0.6</v>
       </c>
       <c r="K273" t="n">
-        <v>307.6</v>
+        <v>306.4</v>
       </c>
       <c r="L273" t="n">
-        <v>19.4</v>
+        <v>20</v>
       </c>
       <c r="M273" t="n">
-        <v>-17.8</v>
+        <v>-18.1</v>
       </c>
       <c r="N273" t="n">
         <v>310.7</v>
       </c>
       <c r="O273" t="n">
-        <v>-1</v>
+        <v>-1.4</v>
       </c>
       <c r="P273" t="n">
-        <v>1064.9</v>
+        <v>1061.6</v>
       </c>
       <c r="Q273" t="n">
-        <v>-41.3</v>
+        <v>-41.5</v>
       </c>
       <c r="R273" t="n">
         <v>1064.2</v>
       </c>
       <c r="S273" t="n">
-        <v>0.1</v>
+        <v>-0.2</v>
       </c>
       <c r="T273" t="n">
-        <v>989.8</v>
+        <v>986.4</v>
       </c>
       <c r="U273" t="n">
         <v>-7.1</v>
@@ -27091,13 +27091,13 @@
         <v>995.7</v>
       </c>
       <c r="W273" t="n">
-        <v>-0.6</v>
+        <v>-0.9</v>
       </c>
       <c r="X273" t="n">
         <v>1873.4</v>
       </c>
       <c r="Y273" t="n">
-        <v>89.3</v>
+        <v>89.90000000000001</v>
       </c>
       <c r="Z273" t="n">
         <v>2003.7</v>

</xml_diff>